<commit_message>
Add household view (Janey + Michael)
- Extend spreadsheet with Michael's inputs (State Pension GBP241/wk from Nov 2039
  ~ GBP12,532/yr, plus editable placeholders for his pot and contributions) and a
  new Household tab combining both, with PLSA couple benchmarks
- Add 06-household-view.md: steady-state household income ~GBP26,800/yr (above the
  couple 'Minimum'; the gap to 'Moderate' is Michael's private pension to add)
- Link the new section from the project README

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ND8Ven1nq7f8ikX2u4rGP4
</commit_message>
<xml_diff>
--- a/janeys-pension-plan/janeys-pension-projections.xlsx
+++ b/janeys-pension-plan/janeys-pension-projections.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Inputs" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Projection" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Retirement income" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Household" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,9 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="£#,##0"/>
+    <numFmt numFmtId="166" formatCode="£#,##0;(£#,##0)"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -120,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -149,6 +151,8 @@
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -514,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -854,6 +858,147 @@
       <c r="C32" s="2" t="inlineStr">
         <is>
           <t>TO TRACE — Teachers' Pension Scheme or LGPS, ~1998–2002. Small but guaranteed &amp; inflation-linked. Request a deferred-benefit statement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Michael (for the household view)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Michael's current age</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="n">
+        <v>53</v>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Inferred from a State Pension date of Nov 2039 (≈ age 67 → born ~late 1972). Adjust if needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Michael's target retirement age</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="n">
+        <v>65</v>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Assumed 65 to match Janey — change to Michael's actual plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Michael's years of contributions (to retirement)</t>
+        </is>
+      </c>
+      <c r="B37" s="4">
+        <f>B36-B35</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Michael's State Pension per week (£)</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="n">
+        <v>241</v>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>From Michael's forecast: £241/week starting Nov 2039.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>Michael's State Pension per year (£)</t>
+        </is>
+      </c>
+      <c r="B39" s="10">
+        <f>B38*52</f>
+        <v>12532</v>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>£241 × 52. Starts Nov 2039 (~age 67).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Michael's existing pension pot today (£)</t>
+        </is>
+      </c>
+      <c r="B40" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>FILL IN — total value of Michael's DC pension pot(s) today.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Michael's gross annual contribution (£)</t>
+        </is>
+      </c>
+      <c r="B41" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>FILL IN — employee + employer + tax relief going in per year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>Michael's pot at retirement (£)</t>
+        </is>
+      </c>
+      <c r="B42" s="10">
+        <f>FV(B23,B37,-B41,-B40,1)</f>
+        <v>0</v>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Grown at the central net rate. Uses the shared growth/charge assumptions above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Michael's drawdown income / yr (£)</t>
+        </is>
+      </c>
+      <c r="B43" s="8">
+        <f>B42*B26</f>
+        <v>0</v>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>~4% of his pot per year.</t>
         </is>
       </c>
     </row>
@@ -1563,4 +1708,268 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Household retirement income — Janey + Michael</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Steady state: both retired and both State Pensions in payment (from ~2039–2040). Fill Michael's pot &amp; contributions on the Inputs tab to complete his private pension.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Annual income (steady state)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>Janey</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>Michael</t>
+        </is>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>Household</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>Private pension (drawdown ~4%)</t>
+        </is>
+      </c>
+      <c r="B6" s="17">
+        <f>'Retirement income'!B14</f>
+        <v>2327.027511</v>
+      </c>
+      <c r="C6" s="17">
+        <f>Inputs!B43</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="18">
+        <f>B6+C6</f>
+        <v>2327.027511</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>Defined-benefit pension</t>
+        </is>
+      </c>
+      <c r="B7" s="17">
+        <f>Inputs!B32</f>
+        <v>0</v>
+      </c>
+      <c r="C7" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="18">
+        <f>B7+C7</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>State Pension</t>
+        </is>
+      </c>
+      <c r="B8" s="17">
+        <f>Inputs!B31</f>
+        <v>11973</v>
+      </c>
+      <c r="C8" s="17">
+        <f>Inputs!B39</f>
+        <v>12532</v>
+      </c>
+      <c r="D8" s="18">
+        <f>B8+C8</f>
+        <v>24505</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="22" t="inlineStr">
+        <is>
+          <t>Total annual income</t>
+        </is>
+      </c>
+      <c r="B9" s="23">
+        <f>SUM(B6:B8)</f>
+        <v>14300.027511</v>
+      </c>
+      <c r="C9" s="23">
+        <f>SUM(C6:C8)</f>
+        <v>12532</v>
+      </c>
+      <c r="D9" s="23">
+        <f>SUM(D6:D8)</f>
+        <v>26832.027511</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>≈ per month</t>
+        </is>
+      </c>
+      <c r="D10" s="8">
+        <f>D9/12</f>
+        <v>2236.002293</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Against PLSA couple benchmarks (today's money)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>Couple / yr</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>Household vs benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Minimum</t>
+        </is>
+      </c>
+      <c r="B14" s="24" t="n">
+        <v>22400</v>
+      </c>
+      <c r="C14" s="25">
+        <f>D9-B14</f>
+        <v>4432.027511</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="B15" s="24" t="n">
+        <v>43100</v>
+      </c>
+      <c r="C15" s="25">
+        <f>D9-B15</f>
+        <v>-16267.972489</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Comfortable</t>
+        </is>
+      </c>
+      <c r="B16" s="24" t="n">
+        <v>59000</v>
+      </c>
+      <c r="C16" s="25">
+        <f>D9-B16</f>
+        <v>-32167.972489</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>PLSA couple figures are illustrative — verify current values at retirementlivingstandards.org.uk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>• Private-pension (drawdown) figures are in FUTURE money; State Pension &amp; DB are in today's money — treat the total as indicative.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>• Timing: Michael's State Pension starts Nov 2039; Janey's at age 67 (~2040). Each has a short gap between retiring at 65 and their State Pension starting — plan those bridge years.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>• Michael's private pension shows £0 until his pot and contributions are entered on the Inputs tab (cells B41, B42).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>• The £500k mortgage-free home is a household asset, not counted as income here — it can support later-life options (e.g. downsizing).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>• This is planning material, not regulated financial advice.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Incorporate Janey's confirmed Teachers' Pension
From Janey's deferred Teachers' Pension benefit statement (identifiers kept
out of the repo for privacy):
- 80th Final Salary: GBP6,981.65/yr unreduced from age 60 + GBP20,944.98 tax-free
  lump sum; Career Average GBP103.48/yr from 67; total GBP7,085.13/yr, index-linked
- This largely solves the pre-State-Pension income bridge (income from age 60)

Model updates:
- Set Janey's DB to GBP6,982; added a Teachers' Pension detail block on Inputs
- Correct Michael's age to 57 (spouse DOB 01/07/1969) and flag the Nov 2039
  State Pension date to confirm
- Household steady-state income now ~GBP33,800/yr (~GBP2,818/mo): above the couple
  'Minimum', ~GBP9.3k short of 'Moderate' before Michael's private pension
- Refresh current-position, strategy, projections, household and checklist docs

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ND8Ven1nq7f8ikX2u4rGP4
</commit_message>
<xml_diff>
--- a/janeys-pension-plan/janeys-pension-projections.xlsx
+++ b/janeys-pension-plan/janeys-pension-projections.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -849,15 +849,15 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>Deferred DB (school) pension per year (£)</t>
-        </is>
-      </c>
-      <c r="B32" s="11" t="n">
-        <v>0</v>
+          <t>Janey's Teachers' Pension per year (£)</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="n">
+        <v>6981.65</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>TO TRACE — Teachers' Pension Scheme or LGPS, ~1998–2002. Small but guaranteed &amp; inflation-linked. Request a deferred-benefit statement.</t>
+          <t>Teachers' Pension (deferred, 19 Sep 2026): £6,981.65 from the 80th Final Salary section, payable UNREDUCED from age 60. Index-linked. See the detail block below.</t>
         </is>
       </c>
     </row>
@@ -875,11 +875,11 @@
         </is>
       </c>
       <c r="B35" s="6" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Inferred from a State Pension date of Nov 2039 (≈ age 67 → born ~late 1972). Adjust if needed.</t>
+          <t>From DOB 01/07/1969 (spouse DOB on Janey's TP statement) → age 57 in 2026. Adjust if wrong.</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="B37" s="4">
         <f>B36-B35</f>
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="38">
@@ -936,7 +936,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>£241 × 52. Starts Nov 2039 (~age 67).</t>
+          <t>£241 × 52. Assumed to start Nov 2039 (per instruction). NOTE: a 1969 DOB would normally mean a State Pension age ~2036–37, so confirm this date at gov.uk/check-state-pension.</t>
         </is>
       </c>
     </row>
@@ -999,6 +999,80 @@
       <c r="C43" s="2" t="inlineStr">
         <is>
           <t>~4% of his pot per year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Janey's Teachers' Pension — detail (deferred, 19 Sep 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>80th Final Salary pension — NPA 60 (from Nov 2032)</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="n">
+        <v>6981.65</v>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Payable UNREDUCED from age 60. Index-linked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Automatic tax-free lump sum (with the 80th pension)</t>
+        </is>
+      </c>
+      <c r="B47" s="8" t="n">
+        <v>20944.98</v>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>One-off, tax-free, from age 60. 3× the pension.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Career Average pension — NPA 67 (from Nov 2039)</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="n">
+        <v>103.48</v>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Small; starts at 67.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Total annual Teachers' Pension from age 67</t>
+        </is>
+      </c>
+      <c r="B49" s="8" t="n">
+        <v>7085.13</v>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>£6,981.65 + £103.48. Both index-linked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Service: 8 yr 288 days · Avg salary ~£39,723 · figures grow with inflation to retirement.</t>
         </is>
       </c>
     </row>
@@ -1627,11 +1701,11 @@
       </c>
       <c r="B20" s="17">
         <f>Inputs!B32</f>
-        <v>0</v>
+        <v>6981.65</v>
       </c>
       <c r="C20" s="17">
         <f>Inputs!B32</f>
-        <v>0</v>
+        <v>6981.65</v>
       </c>
     </row>
     <row r="21">
@@ -1656,11 +1730,11 @@
       </c>
       <c r="B22" s="23">
         <f>SUM(B19:B21)</f>
-        <v>2327.027511</v>
+        <v>9308.677511</v>
       </c>
       <c r="C22" s="23">
         <f>SUM(C19:C21)</f>
-        <v>14300.027511</v>
+        <v>21281.677511</v>
       </c>
     </row>
     <row r="24">
@@ -1687,21 +1761,21 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>2. Trace the 1998–2002 school DB pension and get a deferred statement.</t>
+          <t>2. Teachers' Pension is confirmed: £6,982/yr + £20,945 tax-free lump sum from AGE 60 — this covers the pre-State-Pension years well.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>3. Plan the 65→67 income bridge (private pension / husband's income / savings).</t>
+          <t>3. Decide when to take the Teachers' 80th pension (age 60 unreduced) vs. the personal pot vs. State Pension at 67.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>4. Consider whether the husband can contribute more, or use ISAs, for the household.</t>
+          <t>4. Consider whether Michael can contribute more, or use ISAs, for the household.</t>
         </is>
       </c>
     </row>
@@ -1795,14 +1869,14 @@
       </c>
       <c r="B7" s="17">
         <f>Inputs!B32</f>
-        <v>0</v>
+        <v>6981.65</v>
       </c>
       <c r="C7" s="18" t="n">
         <v>0</v>
       </c>
       <c r="D7" s="18">
         <f>B7+C7</f>
-        <v>0</v>
+        <v>6981.65</v>
       </c>
     </row>
     <row r="8">
@@ -1832,7 +1906,7 @@
       </c>
       <c r="B9" s="23">
         <f>SUM(B6:B8)</f>
-        <v>14300.027511</v>
+        <v>21281.677511</v>
       </c>
       <c r="C9" s="23">
         <f>SUM(C6:C8)</f>
@@ -1840,7 +1914,7 @@
       </c>
       <c r="D9" s="23">
         <f>SUM(D6:D8)</f>
-        <v>26832.027511</v>
+        <v>33813.677511</v>
       </c>
     </row>
     <row r="10">
@@ -1851,7 +1925,7 @@
       </c>
       <c r="D10" s="8">
         <f>D9/12</f>
-        <v>2236.002293</v>
+        <v>2817.806459</v>
       </c>
     </row>
     <row r="12">
@@ -1889,7 +1963,7 @@
       </c>
       <c r="C14" s="25">
         <f>D9-B14</f>
-        <v>4432.027511</v>
+        <v>11413.677511</v>
       </c>
     </row>
     <row r="15">
@@ -1903,7 +1977,7 @@
       </c>
       <c r="C15" s="25">
         <f>D9-B15</f>
-        <v>-16267.972489</v>
+        <v>-9286.322489</v>
       </c>
     </row>
     <row r="16">
@@ -1917,7 +1991,7 @@
       </c>
       <c r="C16" s="25">
         <f>D9-B16</f>
-        <v>-32167.972489</v>
+        <v>-25186.322489</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
Add Michael's pension pot to the household view
From Michael's documents (account numbers/identifiers kept out of the repo):
- Aegon SIPP ~GBP221,974 (consolidated from Scottish Equitable; DC, no safeguarded
  benefits; DOB 02/07/1969 -> age 57)
- 10% salary-sacrifice into a NEST pension since Apr 2025 (salary not yet known)

Model updates:
- Set Michael's existing pot to GBP221,974 (grows to ~GBP315,670 by 65, existing pot only)
- Fix household total cached value to include Michael's drawdown
- Household steady-state income now ~GBP46,440/yr (~GBP3,870/mo): above the couple
  'Moderate' benchmark, ~GBP12,560 short of 'Comfortable' before ongoing contributions
- Refresh current-position and household docs; note NEST pot and salary still to add

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ND8Ven1nq7f8ikX2u4rGP4
</commit_message>
<xml_diff>
--- a/janeys-pension-plan/janeys-pension-projections.xlsx
+++ b/janeys-pension-plan/janeys-pension-projections.xlsx
@@ -879,7 +879,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>From DOB 01/07/1969 (spouse DOB on Janey's TP statement) → age 57 in 2026. Adjust if wrong.</t>
+          <t>From DOB 02/07/1969 (Aegon transfer authority) → age 57 in 2026.</t>
         </is>
       </c>
     </row>
@@ -946,12 +946,12 @@
           <t>Michael's existing pension pot today (£)</t>
         </is>
       </c>
-      <c r="B40" s="11" t="n">
-        <v>0</v>
+      <c r="B40" s="7" t="n">
+        <v>221974.07</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>FILL IN — total value of Michael's DC pension pot(s) today.</t>
+          <t>Aegon SIPP — £221,974.07 consolidated from Scottish Equitable (transfer authority, Jun 2024). Excludes his newer NEST pot (current employer) — value unknown, add when known.</t>
         </is>
       </c>
     </row>
@@ -966,7 +966,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>FILL IN — employee + employer + tax relief going in per year.</t>
+          <t>TO ADD — 10% salary sacrifice into NEST + employer top-up (since Apr 2025). Needs Michael's salary to quantify. Left at £0 for now, so the pot below is 'existing pot only, no new contributions'.</t>
         </is>
       </c>
     </row>
@@ -978,7 +978,7 @@
       </c>
       <c r="B42" s="10">
         <f>FV(B23,B37,-B41,-B40,1)</f>
-        <v>0</v>
+        <v>315669.460981</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
@@ -994,7 +994,7 @@
       </c>
       <c r="B43" s="8">
         <f>B42*B26</f>
-        <v>0</v>
+        <v>12626.778439</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
@@ -1854,11 +1854,11 @@
       </c>
       <c r="C6" s="17">
         <f>Inputs!B43</f>
-        <v>0</v>
+        <v>12626.778439</v>
       </c>
       <c r="D6" s="18">
         <f>B6+C6</f>
-        <v>2327.027511</v>
+        <v>14953.80595</v>
       </c>
     </row>
     <row r="7">
@@ -1910,11 +1910,11 @@
       </c>
       <c r="C9" s="23">
         <f>SUM(C6:C8)</f>
-        <v>12532</v>
+        <v>25158.778439</v>
       </c>
       <c r="D9" s="23">
         <f>SUM(D6:D8)</f>
-        <v>33813.677511</v>
+        <v>46440.45595</v>
       </c>
     </row>
     <row r="10">
@@ -1925,7 +1925,7 @@
       </c>
       <c r="D10" s="8">
         <f>D9/12</f>
-        <v>2817.806459</v>
+        <v>3870.037996</v>
       </c>
     </row>
     <row r="12">
@@ -1963,7 +1963,7 @@
       </c>
       <c r="C14" s="25">
         <f>D9-B14</f>
-        <v>11413.677511</v>
+        <v>24040.45595</v>
       </c>
     </row>
     <row r="15">
@@ -1977,7 +1977,7 @@
       </c>
       <c r="C15" s="25">
         <f>D9-B15</f>
-        <v>-9286.322489</v>
+        <v>3340.45595</v>
       </c>
     </row>
     <row r="16">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="C16" s="25">
         <f>D9-B16</f>
-        <v>-25186.322489</v>
+        <v>-12559.54405</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
Add Michael's salary and contributions; household reaches 'Comfortable'
From Michael's payslip (identifiers kept out of the repo):
- Salary ~GBP171k at One Air Ltd (OPS); ~GBP32,490/yr into pension (19% of salary via
  salary sacrifice, incl. his 10% employee sacrifice)

Model updates:
- Set Michael's contribution to GBP32,490/yr -> pot grows to ~GBP634,140 by 65
- Household steady-state income now ~GBP59,180/yr (~GBP4,932/mo): at the couple
  'Comfortable' PLSA standard (conservative reading; ~GBP49,590/yr contributions
  would be higher still)
- Add Annual Allowance and retirement-tax notes; refresh current-position/household docs
- Remaining: Michael's NEST pot value and State Pension date

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ND8Ven1nq7f8ikX2u4rGP4
</commit_message>
<xml_diff>
--- a/janeys-pension-plan/janeys-pension-projections.xlsx
+++ b/janeys-pension-plan/janeys-pension-projections.xlsx
@@ -961,12 +961,12 @@
           <t>Michael's gross annual contribution (£)</t>
         </is>
       </c>
-      <c r="B41" s="11" t="n">
-        <v>0</v>
+      <c r="B41" s="7" t="n">
+        <v>32490</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>TO ADD — 10% salary sacrifice into NEST + employer top-up (since Apr 2025). Needs Michael's salary to quantify. Left at £0 for now, so the pot below is 'existing pot only, no new contributions'.</t>
+          <t>£2,707.50/mo employer pension × 12 (19% of £171k salary; includes his 10% salary sacrifice). If the £1,425/mo sacrifice is ON TOP, use £49,590. Well within the £60k Annual Allowance.</t>
         </is>
       </c>
     </row>
@@ -978,7 +978,7 @@
       </c>
       <c r="B42" s="10">
         <f>FV(B23,B37,-B41,-B40,1)</f>
-        <v>315669.460981</v>
+        <v>634140.15236</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
@@ -994,7 +994,7 @@
       </c>
       <c r="B43" s="8">
         <f>B42*B26</f>
-        <v>12626.778439</v>
+        <v>25365.606094</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
@@ -1854,11 +1854,11 @@
       </c>
       <c r="C6" s="17">
         <f>Inputs!B43</f>
-        <v>12626.778439</v>
+        <v>25365.606094</v>
       </c>
       <c r="D6" s="18">
         <f>B6+C6</f>
-        <v>14953.80595</v>
+        <v>27692.633606</v>
       </c>
     </row>
     <row r="7">
@@ -1910,11 +1910,11 @@
       </c>
       <c r="C9" s="23">
         <f>SUM(C6:C8)</f>
-        <v>25158.778439</v>
+        <v>37897.606094</v>
       </c>
       <c r="D9" s="23">
         <f>SUM(D6:D8)</f>
-        <v>46440.45595</v>
+        <v>59179.283606</v>
       </c>
     </row>
     <row r="10">
@@ -1925,7 +1925,7 @@
       </c>
       <c r="D10" s="8">
         <f>D9/12</f>
-        <v>3870.037996</v>
+        <v>4931.606967</v>
       </c>
     </row>
     <row r="12">
@@ -1963,7 +1963,7 @@
       </c>
       <c r="C14" s="25">
         <f>D9-B14</f>
-        <v>24040.45595</v>
+        <v>36779.283606</v>
       </c>
     </row>
     <row r="15">
@@ -1977,7 +1977,7 @@
       </c>
       <c r="C15" s="25">
         <f>D9-B15</f>
-        <v>3340.45595</v>
+        <v>16079.283606</v>
       </c>
     </row>
     <row r="16">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="C16" s="25">
         <f>D9-B16</f>
-        <v>-12559.54405</v>
+        <v>179.283606</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
Add Michael's RAF (AFPS 75) preserved pension to the household view
- RAF service 1990-98 (8 yrs, Sergeant, aircrew): left before the 22-year point, so
  a preserved AFPS 75 pension payable from age 60 + ~3x tax-free lump sum, index-linked
- Estimate ~GBP5,340/yr + ~GBP16,020 lump sum (8/22 of a Sgt's ~GBP14,684 22-year pension;
  aircrew rates higher, so likely more - official forecast recommended)
- Add AFPS 75 inputs and include Michael's service pension in the Household tab
- Household steady-state income now ~GBP64,519/yr (~GBP5,377/mo): ~GBP5,500 above the
  couple 'Comfortable' standard, plus ~GBP37k combined tax-free lump sums at age 60
- Confirmed Michael's contributions from the re-sent payment advice (GBP32,490/yr total)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ND8Ven1nq7f8ikX2u4rGP4
</commit_message>
<xml_diff>
--- a/janeys-pension-plan/janeys-pension-projections.xlsx
+++ b/janeys-pension-plan/janeys-pension-projections.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C50"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1073,6 +1073,43 @@
       <c r="A50" s="2" t="inlineStr">
         <is>
           <t>Service: 8 yr 288 days · Avg salary ~£39,723 · figures grow with inflation to retirement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Michael's RAF pension (AFPS 75) — estimate</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>AFPS 75 preserved pension per year (£)</t>
+        </is>
+      </c>
+      <c r="B53" s="11" t="n">
+        <v>5340</v>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>ESTIMATE — RAF 1990–98 (8 yrs), Sgt. ~8/22 of a Sgt's 22-yr pension (~£14,684) ≈ £5,340. Aircrew rates were higher, so likely more. GET AN OFFICIAL FORECAST from Veterans UK / DBS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>AFPS 75 tax-free lump sum (£)</t>
+        </is>
+      </c>
+      <c r="B54" s="11" t="n">
+        <v>16020</v>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>≈ 3 × the annual pension, tax-free. Payable with the pension from AGE 60. Index-linked (CPI).</t>
         </is>
       </c>
     </row>
@@ -1864,19 +1901,20 @@
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>Defined-benefit pension</t>
+          <t>DB / service pension (Teachers' · RAF)</t>
         </is>
       </c>
       <c r="B7" s="17">
         <f>Inputs!B32</f>
         <v>6981.65</v>
       </c>
-      <c r="C7" s="18" t="n">
-        <v>0</v>
+      <c r="C7" s="17">
+        <f>Inputs!B53</f>
+        <v>5340</v>
       </c>
       <c r="D7" s="18">
         <f>B7+C7</f>
-        <v>6981.65</v>
+        <v>12321.65</v>
       </c>
     </row>
     <row r="8">
@@ -1910,11 +1948,11 @@
       </c>
       <c r="C9" s="23">
         <f>SUM(C6:C8)</f>
-        <v>37897.606094</v>
+        <v>43237.606094</v>
       </c>
       <c r="D9" s="23">
         <f>SUM(D6:D8)</f>
-        <v>59179.283606</v>
+        <v>64519.283606</v>
       </c>
     </row>
     <row r="10">
@@ -1925,7 +1963,7 @@
       </c>
       <c r="D10" s="8">
         <f>D9/12</f>
-        <v>4931.606967</v>
+        <v>5376.606967</v>
       </c>
     </row>
     <row r="12">
@@ -1963,7 +2001,7 @@
       </c>
       <c r="C14" s="25">
         <f>D9-B14</f>
-        <v>36779.283606</v>
+        <v>42119.283606</v>
       </c>
     </row>
     <row r="15">
@@ -1977,7 +2015,7 @@
       </c>
       <c r="C15" s="25">
         <f>D9-B15</f>
-        <v>16079.283606</v>
+        <v>21419.283606</v>
       </c>
     </row>
     <row r="16">
@@ -1991,7 +2029,7 @@
       </c>
       <c r="C16" s="25">
         <f>D9-B16</f>
-        <v>179.283606</v>
+        <v>5519.283606</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
Confirm DOBs and resolve State Pension dates
- Michael DOB 02/07/1969 -> State Pension age 67 from ~Jul 2036 (the earlier
  'Nov 2039' was Janey's date)
- Janey DOB 05/11/1972 -> State Pension age 67 from 05/11/2039
- Update spreadsheet notes and household/current-position docs; totals unchanged

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ND8Ven1nq7f8ikX2u4rGP4
</commit_message>
<xml_diff>
--- a/janeys-pension-plan/janeys-pension-projections.xlsx
+++ b/janeys-pension-plan/janeys-pension-projections.xlsx
@@ -583,7 +583,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Born ~1972–73 → State Pension age is 67, not 65. Confirm at gov.uk/state-pension-age.</t>
+          <t>DOB 05/11/1972 → State Pension age 67, payable from 05/11/2039 (not 65).</t>
         </is>
       </c>
     </row>
@@ -879,7 +879,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>From DOB 02/07/1969 (Aegon transfer authority) → age 57 in 2026.</t>
+          <t>DOB 02/07/1969 (confirmed) → age 57 in 2026.</t>
         </is>
       </c>
     </row>
@@ -936,7 +936,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>£241 × 52. Assumed to start Nov 2039 (per instruction). NOTE: a 1969 DOB would normally mean a State Pension age ~2036–37, so confirm this date at gov.uk/check-state-pension.</t>
+          <t>£241 × 52. DOB 02/07/1969 → State Pension age 67, payable from ~02/07/2036 (earlier than the Nov 2039 first assumed). Confirm the amount at gov.uk/check-state-pension.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add year-by-year Timeline tab
- New Timeline tab: household income year by year (2026-2044) as each stream
  switches on (RAF/Teachers' at 60, drawdown at 65, State Pensions at 67), with
  lump-sum events; steady state ~GBP64,519/yr from 2039, matching the Household tab
- Formula-driven off the Inputs tab (recalculates on edit)
- Document the timeline in 06-household-view.md and note the tab in the READMEs

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ND8Ven1nq7f8ikX2u4rGP4
</commit_message>
<xml_diff>
--- a/janeys-pension-plan/janeys-pension-projections.xlsx
+++ b/janeys-pension-plan/janeys-pension-projections.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Projection" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Retirement income" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Household" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Timeline" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -122,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -153,6 +154,8 @@
     <xf numFmtId="165" fontId="6" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2084,4 +2087,1041 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Year-by-year household income (today's money, indicative)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Each stream switches on at the right age (service pensions 60, retirement/drawdown 65, State Pension 67). Amounts as modelled on the other tabs; first year of each may be part-year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Mike</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Jane</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>Mike RAF</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>Mike pot</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>Mike State</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>Jane Tchr</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>Jane pot</t>
+        </is>
+      </c>
+      <c r="I4" s="15" t="inlineStr">
+        <is>
+          <t>Jane State</t>
+        </is>
+      </c>
+      <c r="J4" s="15" t="inlineStr">
+        <is>
+          <t>Household /yr</t>
+        </is>
+      </c>
+      <c r="K4" s="15" t="inlineStr">
+        <is>
+          <t>Lump sums</t>
+        </is>
+      </c>
+      <c r="L4" s="15" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B5" s="16">
+        <f>A5-1969</f>
+        <v>57</v>
+      </c>
+      <c r="C5" s="16">
+        <f>A5-1972</f>
+        <v>54</v>
+      </c>
+      <c r="D5" s="18">
+        <f>IF(B5&gt;=60,Inputs!B53,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E5" s="18">
+        <f>IF(B5&gt;=Inputs!B36,Inputs!B43,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="18">
+        <f>IF(B5&gt;=67,Inputs!B39,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G5" s="18">
+        <f>IF(C5&gt;=60,Inputs!B32,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H5" s="18">
+        <f>IF(C5&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I5" s="18">
+        <f>IF(C5&gt;=67,Inputs!B31,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J5" s="23">
+        <f>SUM(D5:I5)</f>
+        <v>0</v>
+      </c>
+      <c r="K5" s="18">
+        <f>IF(B5=60,Inputs!B54,0)+IF(C5=60,Inputs!B47,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L5" s="26" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B6" s="16">
+        <f>A6-1969</f>
+        <v>58</v>
+      </c>
+      <c r="C6" s="16">
+        <f>A6-1972</f>
+        <v>55</v>
+      </c>
+      <c r="D6" s="18">
+        <f>IF(B6&gt;=60,Inputs!B53,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E6" s="18">
+        <f>IF(B6&gt;=Inputs!B36,Inputs!B43,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="18">
+        <f>IF(B6&gt;=67,Inputs!B39,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="18">
+        <f>IF(C6&gt;=60,Inputs!B32,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="18">
+        <f>IF(C6&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I6" s="18">
+        <f>IF(C6&gt;=67,Inputs!B31,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J6" s="23">
+        <f>SUM(D6:I6)</f>
+        <v>0</v>
+      </c>
+      <c r="K6" s="18">
+        <f>IF(B6=60,Inputs!B54,0)+IF(C6=60,Inputs!B47,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L6" s="26" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="n">
+        <v>2028</v>
+      </c>
+      <c r="B7" s="16">
+        <f>A7-1969</f>
+        <v>59</v>
+      </c>
+      <c r="C7" s="16">
+        <f>A7-1972</f>
+        <v>56</v>
+      </c>
+      <c r="D7" s="18">
+        <f>IF(B7&gt;=60,Inputs!B53,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E7" s="18">
+        <f>IF(B7&gt;=Inputs!B36,Inputs!B43,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="18">
+        <f>IF(B7&gt;=67,Inputs!B39,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="18">
+        <f>IF(C7&gt;=60,Inputs!B32,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H7" s="18">
+        <f>IF(C7&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I7" s="18">
+        <f>IF(C7&gt;=67,Inputs!B31,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J7" s="23">
+        <f>SUM(D7:I7)</f>
+        <v>0</v>
+      </c>
+      <c r="K7" s="18">
+        <f>IF(B7=60,Inputs!B54,0)+IF(C7=60,Inputs!B47,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L7" s="26" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="n">
+        <v>2029</v>
+      </c>
+      <c r="B8" s="16">
+        <f>A8-1969</f>
+        <v>60</v>
+      </c>
+      <c r="C8" s="16">
+        <f>A8-1972</f>
+        <v>57</v>
+      </c>
+      <c r="D8" s="18">
+        <f>IF(B8&gt;=60,Inputs!B53,0)</f>
+        <v>5340</v>
+      </c>
+      <c r="E8" s="18">
+        <f>IF(B8&gt;=Inputs!B36,Inputs!B43,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="18">
+        <f>IF(B8&gt;=67,Inputs!B39,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="18">
+        <f>IF(C8&gt;=60,Inputs!B32,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H8" s="18">
+        <f>IF(C8&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I8" s="18">
+        <f>IF(C8&gt;=67,Inputs!B31,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J8" s="23">
+        <f>SUM(D8:I8)</f>
+        <v>5340</v>
+      </c>
+      <c r="K8" s="18">
+        <f>IF(B8=60,Inputs!B54,0)+IF(C8=60,Inputs!B47,0)</f>
+        <v>16020</v>
+      </c>
+      <c r="L8" s="27" t="inlineStr">
+        <is>
+          <t>Mike 60 → RAF pension + lump sum</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="n">
+        <v>2030</v>
+      </c>
+      <c r="B9" s="16">
+        <f>A9-1969</f>
+        <v>61</v>
+      </c>
+      <c r="C9" s="16">
+        <f>A9-1972</f>
+        <v>58</v>
+      </c>
+      <c r="D9" s="18">
+        <f>IF(B9&gt;=60,Inputs!B53,0)</f>
+        <v>5340</v>
+      </c>
+      <c r="E9" s="18">
+        <f>IF(B9&gt;=Inputs!B36,Inputs!B43,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="18">
+        <f>IF(B9&gt;=67,Inputs!B39,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="18">
+        <f>IF(C9&gt;=60,Inputs!B32,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="18">
+        <f>IF(C9&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I9" s="18">
+        <f>IF(C9&gt;=67,Inputs!B31,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J9" s="23">
+        <f>SUM(D9:I9)</f>
+        <v>5340</v>
+      </c>
+      <c r="K9" s="18">
+        <f>IF(B9=60,Inputs!B54,0)+IF(C9=60,Inputs!B47,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L9" s="26" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="n">
+        <v>2031</v>
+      </c>
+      <c r="B10" s="16">
+        <f>A10-1969</f>
+        <v>62</v>
+      </c>
+      <c r="C10" s="16">
+        <f>A10-1972</f>
+        <v>59</v>
+      </c>
+      <c r="D10" s="18">
+        <f>IF(B10&gt;=60,Inputs!B53,0)</f>
+        <v>5340</v>
+      </c>
+      <c r="E10" s="18">
+        <f>IF(B10&gt;=Inputs!B36,Inputs!B43,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="18">
+        <f>IF(B10&gt;=67,Inputs!B39,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="18">
+        <f>IF(C10&gt;=60,Inputs!B32,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H10" s="18">
+        <f>IF(C10&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I10" s="18">
+        <f>IF(C10&gt;=67,Inputs!B31,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J10" s="23">
+        <f>SUM(D10:I10)</f>
+        <v>5340</v>
+      </c>
+      <c r="K10" s="18">
+        <f>IF(B10=60,Inputs!B54,0)+IF(C10=60,Inputs!B47,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L10" s="26" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="n">
+        <v>2032</v>
+      </c>
+      <c r="B11" s="16">
+        <f>A11-1969</f>
+        <v>63</v>
+      </c>
+      <c r="C11" s="16">
+        <f>A11-1972</f>
+        <v>60</v>
+      </c>
+      <c r="D11" s="18">
+        <f>IF(B11&gt;=60,Inputs!B53,0)</f>
+        <v>5340</v>
+      </c>
+      <c r="E11" s="18">
+        <f>IF(B11&gt;=Inputs!B36,Inputs!B43,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="18">
+        <f>IF(B11&gt;=67,Inputs!B39,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="18">
+        <f>IF(C11&gt;=60,Inputs!B32,0)</f>
+        <v>6981.65</v>
+      </c>
+      <c r="H11" s="18">
+        <f>IF(C11&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I11" s="18">
+        <f>IF(C11&gt;=67,Inputs!B31,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J11" s="23">
+        <f>SUM(D11:I11)</f>
+        <v>12321.65</v>
+      </c>
+      <c r="K11" s="18">
+        <f>IF(B11=60,Inputs!B54,0)+IF(C11=60,Inputs!B47,0)</f>
+        <v>20944.98</v>
+      </c>
+      <c r="L11" s="27" t="inlineStr">
+        <is>
+          <t>Jane 60 → Teachers' pension + lump sum</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="n">
+        <v>2033</v>
+      </c>
+      <c r="B12" s="16">
+        <f>A12-1969</f>
+        <v>64</v>
+      </c>
+      <c r="C12" s="16">
+        <f>A12-1972</f>
+        <v>61</v>
+      </c>
+      <c r="D12" s="18">
+        <f>IF(B12&gt;=60,Inputs!B53,0)</f>
+        <v>5340</v>
+      </c>
+      <c r="E12" s="18">
+        <f>IF(B12&gt;=Inputs!B36,Inputs!B43,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F12" s="18">
+        <f>IF(B12&gt;=67,Inputs!B39,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="18">
+        <f>IF(C12&gt;=60,Inputs!B32,0)</f>
+        <v>6981.65</v>
+      </c>
+      <c r="H12" s="18">
+        <f>IF(C12&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I12" s="18">
+        <f>IF(C12&gt;=67,Inputs!B31,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J12" s="23">
+        <f>SUM(D12:I12)</f>
+        <v>12321.65</v>
+      </c>
+      <c r="K12" s="18">
+        <f>IF(B12=60,Inputs!B54,0)+IF(C12=60,Inputs!B47,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L12" s="26" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="n">
+        <v>2034</v>
+      </c>
+      <c r="B13" s="16">
+        <f>A13-1969</f>
+        <v>65</v>
+      </c>
+      <c r="C13" s="16">
+        <f>A13-1972</f>
+        <v>62</v>
+      </c>
+      <c r="D13" s="18">
+        <f>IF(B13&gt;=60,Inputs!B53,0)</f>
+        <v>5340</v>
+      </c>
+      <c r="E13" s="18">
+        <f>IF(B13&gt;=Inputs!B36,Inputs!B43,0)</f>
+        <v>25365.606094</v>
+      </c>
+      <c r="F13" s="18">
+        <f>IF(B13&gt;=67,Inputs!B39,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="18">
+        <f>IF(C13&gt;=60,Inputs!B32,0)</f>
+        <v>6981.65</v>
+      </c>
+      <c r="H13" s="18">
+        <f>IF(C13&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I13" s="18">
+        <f>IF(C13&gt;=67,Inputs!B31,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J13" s="23">
+        <f>SUM(D13:I13)</f>
+        <v>37687.256094</v>
+      </c>
+      <c r="K13" s="18">
+        <f>IF(B13=60,Inputs!B54,0)+IF(C13=60,Inputs!B47,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L13" s="27" t="inlineStr">
+        <is>
+          <t>Mike 65 → retires, draws DC pot</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="n">
+        <v>2035</v>
+      </c>
+      <c r="B14" s="16">
+        <f>A14-1969</f>
+        <v>66</v>
+      </c>
+      <c r="C14" s="16">
+        <f>A14-1972</f>
+        <v>63</v>
+      </c>
+      <c r="D14" s="18">
+        <f>IF(B14&gt;=60,Inputs!B53,0)</f>
+        <v>5340</v>
+      </c>
+      <c r="E14" s="18">
+        <f>IF(B14&gt;=Inputs!B36,Inputs!B43,0)</f>
+        <v>25365.606094</v>
+      </c>
+      <c r="F14" s="18">
+        <f>IF(B14&gt;=67,Inputs!B39,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G14" s="18">
+        <f>IF(C14&gt;=60,Inputs!B32,0)</f>
+        <v>6981.65</v>
+      </c>
+      <c r="H14" s="18">
+        <f>IF(C14&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I14" s="18">
+        <f>IF(C14&gt;=67,Inputs!B31,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J14" s="23">
+        <f>SUM(D14:I14)</f>
+        <v>37687.256094</v>
+      </c>
+      <c r="K14" s="18">
+        <f>IF(B14=60,Inputs!B54,0)+IF(C14=60,Inputs!B47,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L14" s="26" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="n">
+        <v>2036</v>
+      </c>
+      <c r="B15" s="16">
+        <f>A15-1969</f>
+        <v>67</v>
+      </c>
+      <c r="C15" s="16">
+        <f>A15-1972</f>
+        <v>64</v>
+      </c>
+      <c r="D15" s="18">
+        <f>IF(B15&gt;=60,Inputs!B53,0)</f>
+        <v>5340</v>
+      </c>
+      <c r="E15" s="18">
+        <f>IF(B15&gt;=Inputs!B36,Inputs!B43,0)</f>
+        <v>25365.606094</v>
+      </c>
+      <c r="F15" s="18">
+        <f>IF(B15&gt;=67,Inputs!B39,0)</f>
+        <v>12532</v>
+      </c>
+      <c r="G15" s="18">
+        <f>IF(C15&gt;=60,Inputs!B32,0)</f>
+        <v>6981.65</v>
+      </c>
+      <c r="H15" s="18">
+        <f>IF(C15&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I15" s="18">
+        <f>IF(C15&gt;=67,Inputs!B31,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J15" s="23">
+        <f>SUM(D15:I15)</f>
+        <v>50219.256094</v>
+      </c>
+      <c r="K15" s="18">
+        <f>IF(B15=60,Inputs!B54,0)+IF(C15=60,Inputs!B47,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L15" s="27" t="inlineStr">
+        <is>
+          <t>Mike 67 → State Pension starts</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="n">
+        <v>2037</v>
+      </c>
+      <c r="B16" s="16">
+        <f>A16-1969</f>
+        <v>68</v>
+      </c>
+      <c r="C16" s="16">
+        <f>A16-1972</f>
+        <v>65</v>
+      </c>
+      <c r="D16" s="18">
+        <f>IF(B16&gt;=60,Inputs!B53,0)</f>
+        <v>5340</v>
+      </c>
+      <c r="E16" s="18">
+        <f>IF(B16&gt;=Inputs!B36,Inputs!B43,0)</f>
+        <v>25365.606094</v>
+      </c>
+      <c r="F16" s="18">
+        <f>IF(B16&gt;=67,Inputs!B39,0)</f>
+        <v>12532</v>
+      </c>
+      <c r="G16" s="18">
+        <f>IF(C16&gt;=60,Inputs!B32,0)</f>
+        <v>6981.65</v>
+      </c>
+      <c r="H16" s="18">
+        <f>IF(C16&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
+        <v>2327.027511</v>
+      </c>
+      <c r="I16" s="18">
+        <f>IF(C16&gt;=67,Inputs!B31,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J16" s="23">
+        <f>SUM(D16:I16)</f>
+        <v>52546.283606</v>
+      </c>
+      <c r="K16" s="18">
+        <f>IF(B16=60,Inputs!B54,0)+IF(C16=60,Inputs!B47,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L16" s="27" t="inlineStr">
+        <is>
+          <t>Jane 65 → retires, draws DC pot</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="n">
+        <v>2038</v>
+      </c>
+      <c r="B17" s="16">
+        <f>A17-1969</f>
+        <v>69</v>
+      </c>
+      <c r="C17" s="16">
+        <f>A17-1972</f>
+        <v>66</v>
+      </c>
+      <c r="D17" s="18">
+        <f>IF(B17&gt;=60,Inputs!B53,0)</f>
+        <v>5340</v>
+      </c>
+      <c r="E17" s="18">
+        <f>IF(B17&gt;=Inputs!B36,Inputs!B43,0)</f>
+        <v>25365.606094</v>
+      </c>
+      <c r="F17" s="18">
+        <f>IF(B17&gt;=67,Inputs!B39,0)</f>
+        <v>12532</v>
+      </c>
+      <c r="G17" s="18">
+        <f>IF(C17&gt;=60,Inputs!B32,0)</f>
+        <v>6981.65</v>
+      </c>
+      <c r="H17" s="18">
+        <f>IF(C17&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
+        <v>2327.027511</v>
+      </c>
+      <c r="I17" s="18">
+        <f>IF(C17&gt;=67,Inputs!B31,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J17" s="23">
+        <f>SUM(D17:I17)</f>
+        <v>52546.283606</v>
+      </c>
+      <c r="K17" s="18">
+        <f>IF(B17=60,Inputs!B54,0)+IF(C17=60,Inputs!B47,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L17" s="26" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="n">
+        <v>2039</v>
+      </c>
+      <c r="B18" s="16">
+        <f>A18-1969</f>
+        <v>70</v>
+      </c>
+      <c r="C18" s="16">
+        <f>A18-1972</f>
+        <v>67</v>
+      </c>
+      <c r="D18" s="18">
+        <f>IF(B18&gt;=60,Inputs!B53,0)</f>
+        <v>5340</v>
+      </c>
+      <c r="E18" s="18">
+        <f>IF(B18&gt;=Inputs!B36,Inputs!B43,0)</f>
+        <v>25365.606094</v>
+      </c>
+      <c r="F18" s="18">
+        <f>IF(B18&gt;=67,Inputs!B39,0)</f>
+        <v>12532</v>
+      </c>
+      <c r="G18" s="18">
+        <f>IF(C18&gt;=60,Inputs!B32,0)</f>
+        <v>6981.65</v>
+      </c>
+      <c r="H18" s="18">
+        <f>IF(C18&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
+        <v>2327.027511</v>
+      </c>
+      <c r="I18" s="18">
+        <f>IF(C18&gt;=67,Inputs!B31,0)</f>
+        <v>11973</v>
+      </c>
+      <c r="J18" s="23">
+        <f>SUM(D18:I18)</f>
+        <v>64519.283606</v>
+      </c>
+      <c r="K18" s="18">
+        <f>IF(B18=60,Inputs!B54,0)+IF(C18=60,Inputs!B47,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L18" s="27" t="inlineStr">
+        <is>
+          <t>Jane 67 → State Pension starts (all streams on)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="n">
+        <v>2040</v>
+      </c>
+      <c r="B19" s="16">
+        <f>A19-1969</f>
+        <v>71</v>
+      </c>
+      <c r="C19" s="16">
+        <f>A19-1972</f>
+        <v>68</v>
+      </c>
+      <c r="D19" s="18">
+        <f>IF(B19&gt;=60,Inputs!B53,0)</f>
+        <v>5340</v>
+      </c>
+      <c r="E19" s="18">
+        <f>IF(B19&gt;=Inputs!B36,Inputs!B43,0)</f>
+        <v>25365.606094</v>
+      </c>
+      <c r="F19" s="18">
+        <f>IF(B19&gt;=67,Inputs!B39,0)</f>
+        <v>12532</v>
+      </c>
+      <c r="G19" s="18">
+        <f>IF(C19&gt;=60,Inputs!B32,0)</f>
+        <v>6981.65</v>
+      </c>
+      <c r="H19" s="18">
+        <f>IF(C19&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
+        <v>2327.027511</v>
+      </c>
+      <c r="I19" s="18">
+        <f>IF(C19&gt;=67,Inputs!B31,0)</f>
+        <v>11973</v>
+      </c>
+      <c r="J19" s="23">
+        <f>SUM(D19:I19)</f>
+        <v>64519.283606</v>
+      </c>
+      <c r="K19" s="18">
+        <f>IF(B19=60,Inputs!B54,0)+IF(C19=60,Inputs!B47,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L19" s="26" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="n">
+        <v>2041</v>
+      </c>
+      <c r="B20" s="16">
+        <f>A20-1969</f>
+        <v>72</v>
+      </c>
+      <c r="C20" s="16">
+        <f>A20-1972</f>
+        <v>69</v>
+      </c>
+      <c r="D20" s="18">
+        <f>IF(B20&gt;=60,Inputs!B53,0)</f>
+        <v>5340</v>
+      </c>
+      <c r="E20" s="18">
+        <f>IF(B20&gt;=Inputs!B36,Inputs!B43,0)</f>
+        <v>25365.606094</v>
+      </c>
+      <c r="F20" s="18">
+        <f>IF(B20&gt;=67,Inputs!B39,0)</f>
+        <v>12532</v>
+      </c>
+      <c r="G20" s="18">
+        <f>IF(C20&gt;=60,Inputs!B32,0)</f>
+        <v>6981.65</v>
+      </c>
+      <c r="H20" s="18">
+        <f>IF(C20&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
+        <v>2327.027511</v>
+      </c>
+      <c r="I20" s="18">
+        <f>IF(C20&gt;=67,Inputs!B31,0)</f>
+        <v>11973</v>
+      </c>
+      <c r="J20" s="23">
+        <f>SUM(D20:I20)</f>
+        <v>64519.283606</v>
+      </c>
+      <c r="K20" s="18">
+        <f>IF(B20=60,Inputs!B54,0)+IF(C20=60,Inputs!B47,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L20" s="26" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="n">
+        <v>2042</v>
+      </c>
+      <c r="B21" s="16">
+        <f>A21-1969</f>
+        <v>73</v>
+      </c>
+      <c r="C21" s="16">
+        <f>A21-1972</f>
+        <v>70</v>
+      </c>
+      <c r="D21" s="18">
+        <f>IF(B21&gt;=60,Inputs!B53,0)</f>
+        <v>5340</v>
+      </c>
+      <c r="E21" s="18">
+        <f>IF(B21&gt;=Inputs!B36,Inputs!B43,0)</f>
+        <v>25365.606094</v>
+      </c>
+      <c r="F21" s="18">
+        <f>IF(B21&gt;=67,Inputs!B39,0)</f>
+        <v>12532</v>
+      </c>
+      <c r="G21" s="18">
+        <f>IF(C21&gt;=60,Inputs!B32,0)</f>
+        <v>6981.65</v>
+      </c>
+      <c r="H21" s="18">
+        <f>IF(C21&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
+        <v>2327.027511</v>
+      </c>
+      <c r="I21" s="18">
+        <f>IF(C21&gt;=67,Inputs!B31,0)</f>
+        <v>11973</v>
+      </c>
+      <c r="J21" s="23">
+        <f>SUM(D21:I21)</f>
+        <v>64519.283606</v>
+      </c>
+      <c r="K21" s="18">
+        <f>IF(B21=60,Inputs!B54,0)+IF(C21=60,Inputs!B47,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L21" s="26" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="n">
+        <v>2043</v>
+      </c>
+      <c r="B22" s="16">
+        <f>A22-1969</f>
+        <v>74</v>
+      </c>
+      <c r="C22" s="16">
+        <f>A22-1972</f>
+        <v>71</v>
+      </c>
+      <c r="D22" s="18">
+        <f>IF(B22&gt;=60,Inputs!B53,0)</f>
+        <v>5340</v>
+      </c>
+      <c r="E22" s="18">
+        <f>IF(B22&gt;=Inputs!B36,Inputs!B43,0)</f>
+        <v>25365.606094</v>
+      </c>
+      <c r="F22" s="18">
+        <f>IF(B22&gt;=67,Inputs!B39,0)</f>
+        <v>12532</v>
+      </c>
+      <c r="G22" s="18">
+        <f>IF(C22&gt;=60,Inputs!B32,0)</f>
+        <v>6981.65</v>
+      </c>
+      <c r="H22" s="18">
+        <f>IF(C22&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
+        <v>2327.027511</v>
+      </c>
+      <c r="I22" s="18">
+        <f>IF(C22&gt;=67,Inputs!B31,0)</f>
+        <v>11973</v>
+      </c>
+      <c r="J22" s="23">
+        <f>SUM(D22:I22)</f>
+        <v>64519.283606</v>
+      </c>
+      <c r="K22" s="18">
+        <f>IF(B22=60,Inputs!B54,0)+IF(C22=60,Inputs!B47,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L22" s="26" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="n">
+        <v>2044</v>
+      </c>
+      <c r="B23" s="16">
+        <f>A23-1969</f>
+        <v>75</v>
+      </c>
+      <c r="C23" s="16">
+        <f>A23-1972</f>
+        <v>72</v>
+      </c>
+      <c r="D23" s="18">
+        <f>IF(B23&gt;=60,Inputs!B53,0)</f>
+        <v>5340</v>
+      </c>
+      <c r="E23" s="18">
+        <f>IF(B23&gt;=Inputs!B36,Inputs!B43,0)</f>
+        <v>25365.606094</v>
+      </c>
+      <c r="F23" s="18">
+        <f>IF(B23&gt;=67,Inputs!B39,0)</f>
+        <v>12532</v>
+      </c>
+      <c r="G23" s="18">
+        <f>IF(C23&gt;=60,Inputs!B32,0)</f>
+        <v>6981.65</v>
+      </c>
+      <c r="H23" s="18">
+        <f>IF(C23&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
+        <v>2327.027511</v>
+      </c>
+      <c r="I23" s="18">
+        <f>IF(C23&gt;=67,Inputs!B31,0)</f>
+        <v>11973</v>
+      </c>
+      <c r="J23" s="23">
+        <f>SUM(D23:I23)</f>
+        <v>64519.283606</v>
+      </c>
+      <c r="K23" s="18">
+        <f>IF(B23=60,Inputs!B54,0)+IF(C23=60,Inputs!B47,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L23" s="26" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Notes:</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>• Today's-money / real terms: guaranteed pensions (State, Teachers', RAF) are index-linked; drawdown shown flat at the modelled amount.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>• Service pensions (Teachers', RAF) and their tax-free lump sums start at AGE 60 — so income is covered well before the State Pensions begin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>• 'Lump sums' column = one-off tax-free cash that year (RAF at Mike 60, Teachers' at Jane 60). The DC pots' 25% tax-free cash is additional and not shown here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>• Household /yr = sum of all streams live that year. Change any input on the Inputs tab and this recalculates.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add early-retirement comparison tab (Mike 60 vs 62 vs 65)
- New 'Retire 60 vs 65' tab: Michael's pot, drawdown and household income for
  retirement at 60/62/65, formula-driven off the Inputs tab
- Retire 60 -> ~GBP53,500/yr household (above Moderate, ~GBP5.5k short of Comfortable);
  62 -> ~GBP57,650; 65 -> ~GBP64,500. Each extra year worked ~+GBP2,000/yr for life
- Document the comparison in 06-household-view.md and note the tab in the READMEs

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ND8Ven1nq7f8ikX2u4rGP4
</commit_message>
<xml_diff>
--- a/janeys-pension-plan/janeys-pension-projections.xlsx
+++ b/janeys-pension-plan/janeys-pension-projections.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Retirement income" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Household" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Timeline" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Retire 60 vs 65" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -123,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -156,6 +157,8 @@
     <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3124,4 +3127,301 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Michael — retire early? (60 vs 62 vs 65)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Only Michael's DC pot changes with his retirement age (fewer contributions + less growth). RAF, State and Janey's pensions are unchanged. Edit the ages in row 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>Retire at 60</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>Retire at 62</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>Retire at 65</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Michael's retirement age</t>
+        </is>
+      </c>
+      <c r="B5" s="28" t="n">
+        <v>60</v>
+      </c>
+      <c r="C5" s="28" t="n">
+        <v>62</v>
+      </c>
+      <c r="D5" s="28" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>Years of contributions</t>
+        </is>
+      </c>
+      <c r="B6" s="16">
+        <f>B5-Inputs!B35</f>
+        <v>3</v>
+      </c>
+      <c r="C6" s="16">
+        <f>C5-Inputs!B35</f>
+        <v>5</v>
+      </c>
+      <c r="D6" s="16">
+        <f>D5-Inputs!B35</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>Michael's pot at retirement</t>
+        </is>
+      </c>
+      <c r="B7" s="18">
+        <f>FV(Inputs!B23,B6,-Inputs!B41,-Inputs!B40,1)</f>
+        <v>359817.718964</v>
+      </c>
+      <c r="C7" s="18">
+        <f>FV(Inputs!B23,C6,-Inputs!B41,-Inputs!B40,1)</f>
+        <v>462361.886801</v>
+      </c>
+      <c r="D7" s="18">
+        <f>FV(Inputs!B23,D6,-Inputs!B41,-Inputs!B40,1)</f>
+        <v>634140.15236</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Michael's drawdown (~4%/yr)</t>
+        </is>
+      </c>
+      <c r="B8" s="18">
+        <f>B7*Inputs!B26</f>
+        <v>14392.708759</v>
+      </c>
+      <c r="C8" s="18">
+        <f>C7*Inputs!B26</f>
+        <v>18494.475472</v>
+      </c>
+      <c r="D8" s="18">
+        <f>D7*Inputs!B26</f>
+        <v>25365.606094</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>+ RAF pension</t>
+        </is>
+      </c>
+      <c r="B9" s="17">
+        <f>Inputs!B53</f>
+        <v>5340</v>
+      </c>
+      <c r="C9" s="17">
+        <f>Inputs!B53</f>
+        <v>5340</v>
+      </c>
+      <c r="D9" s="17">
+        <f>Inputs!B53</f>
+        <v>5340</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>+ State Pension</t>
+        </is>
+      </c>
+      <c r="B10" s="17">
+        <f>Inputs!B39</f>
+        <v>12532</v>
+      </c>
+      <c r="C10" s="17">
+        <f>Inputs!B39</f>
+        <v>12532</v>
+      </c>
+      <c r="D10" s="17">
+        <f>Inputs!B39</f>
+        <v>12532</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="22" t="inlineStr">
+        <is>
+          <t>Michael's total income /yr</t>
+        </is>
+      </c>
+      <c r="B11" s="29">
+        <f>B8+B9+B10</f>
+        <v>32264.708759</v>
+      </c>
+      <c r="C11" s="29">
+        <f>C8+C9+C10</f>
+        <v>36366.475472</v>
+      </c>
+      <c r="D11" s="29">
+        <f>D8+D9+D10</f>
+        <v>43237.606094</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Janey's total income /yr</t>
+        </is>
+      </c>
+      <c r="B12" s="17">
+        <f>'Household'!B9</f>
+        <v>21281.677511</v>
+      </c>
+      <c r="C12" s="17">
+        <f>'Household'!B9</f>
+        <v>21281.677511</v>
+      </c>
+      <c r="D12" s="17">
+        <f>'Household'!B9</f>
+        <v>21281.677511</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="22" t="inlineStr">
+        <is>
+          <t>Household total /yr</t>
+        </is>
+      </c>
+      <c r="B13" s="23">
+        <f>B11+B12</f>
+        <v>53546.38627</v>
+      </c>
+      <c r="C13" s="23">
+        <f>C11+C12</f>
+        <v>57648.152983</v>
+      </c>
+      <c r="D13" s="23">
+        <f>D11+D12</f>
+        <v>64519.283606</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>≈ per month</t>
+        </is>
+      </c>
+      <c r="B14" s="18">
+        <f>B13/12</f>
+        <v>4462.198856</v>
+      </c>
+      <c r="C14" s="18">
+        <f>C13/12</f>
+        <v>4804.012749</v>
+      </c>
+      <c r="D14" s="18">
+        <f>D13/12</f>
+        <v>5376.606967</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>vs 'Comfortable' (£59,000)</t>
+        </is>
+      </c>
+      <c r="B15" s="25">
+        <f>B13-59000</f>
+        <v>-5453.61373</v>
+      </c>
+      <c r="C15" s="25">
+        <f>C13-59000</f>
+        <v>-1351.847017</v>
+      </c>
+      <c r="D15" s="25">
+        <f>D13-59000</f>
+        <v>5519.283606</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Notes:</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>• Retiring earlier means fewer years of contributions AND less growth, so a smaller pot and lower drawdown for life.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>• It also means giving up salary for those years (~£171k/yr) and funding a LONGER retirement — a 30+ year retirement from age 60 may warrant a more cautious ~3.5% withdrawal rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>• RAF pension (from 60), State Pension (from 67) and Janey's pensions are unchanged by Michael's retirement age.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>• Figures are indicative and in mixed money terms, consistent with the Household tab.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Comfortable-plus scenario tab (with Michael's NEST pot)
- New 'Comfortable-plus' tab: adds Michael's existing NEST pot (current One Air
  pension, separate from the Aegon SIPP) on top of the base household income
- NEST value is an editable estimate (~GBP47k, ~GBP2,707/mo since Apr 2025) in cell B4 -
  replace with the real balance; only the existing balance is added (ongoing
  contributions already counted in the base, so no double-count)
- Household income -> ~GBP67,193/yr (~GBP5,599/mo), ~GBP8,193 above 'Comfortable'
- Document in 06-household-view.md and note the tab in the READMEs

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ND8Ven1nq7f8ikX2u4rGP4
</commit_message>
<xml_diff>
--- a/janeys-pension-plan/janeys-pension-projections.xlsx
+++ b/janeys-pension-plan/janeys-pension-projections.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Household" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Timeline" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Retire 60 vs 65" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Comfortable-plus" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -124,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -159,6 +160,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3424,4 +3426,187 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Comfortable-plus — including Michael's NEST pot</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>NEST = Michael's current One Air pension (since Apr 2025), separate from the £221,974 Aegon SIPP. The value below is an ESTIMATE — replace B4 with the real figure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Michael's NEST pot today (£)</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n">
+        <v>47000</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>ESTIMATE: ~£2,707.50/mo since Apr 2025 ≈ £47k. Replace with the real NEST balance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>NEST pot at 65 (central growth)</t>
+        </is>
+      </c>
+      <c r="B5" s="8">
+        <f>FV(Inputs!B23,Inputs!B37,0,-B4,1)</f>
+        <v>66838.728803</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Existing balance grown to 65. No extra contributions here — ongoing ones are already in the base.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Extra drawdown from NEST (~4%/yr)</t>
+        </is>
+      </c>
+      <c r="B6" s="8">
+        <f>B5*Inputs!B26</f>
+        <v>2673.549152</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>The income the NEST pot adds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Household income — base (Household tab)</t>
+        </is>
+      </c>
+      <c r="B8" s="8">
+        <f>'Household'!D9</f>
+        <v>64519.283606</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>The ~£64,519/yr steady-state total, before NEST.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>+ NEST drawdown</t>
+        </is>
+      </c>
+      <c r="B9" s="8">
+        <f>B6</f>
+        <v>2673.549152</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Household income — Comfortable-plus /yr</t>
+        </is>
+      </c>
+      <c r="B10" s="19">
+        <f>B8+B9</f>
+        <v>67192.832758</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Base + NEST.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>≈ per month</t>
+        </is>
+      </c>
+      <c r="B11" s="8">
+        <f>B10/12</f>
+        <v>5599.40273</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>vs 'Comfortable' (£59,000)</t>
+        </is>
+      </c>
+      <c r="B12" s="30">
+        <f>B10-59000</f>
+        <v>8192.832758</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Notes:</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>• Only the EXISTING NEST balance is added here; the ongoing £32,490/yr contributions are already counted in the base (Household tab).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>• Replace the £47k estimate in B4 with Michael's actual NEST value for an exact figure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>• Both DC pots (Aegon + NEST) also carry 25% tax-free cash at retirement, on top of the lump sums shown elsewhere.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>• Indicative, mixed money terms, consistent with the Household tab.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update Janey's State Pension to GBP12,500 (full payments confirmed)
- Janey's State Pension confirmed at GBP12,500/yr with full payments -> no NI gaps
- Recalculate all tabs: household ~GBP65,046/yr (~GBP5,421/mo), ~GBP6,050 above
  'Comfortable'; Comfortable-plus ~GBP67,720/yr; early-retirement 60/62/65 ->
  ~GBP54,070 / GBP58,175 / GBP65,046
- Update current-position, strategy, projections, household, inputs and checklist
  docs; the State Pension forecast / NI-gap items are now closed

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ND8Ven1nq7f8ikX2u4rGP4
</commit_message>
<xml_diff>
--- a/janeys-pension-plan/janeys-pension-projections.xlsx
+++ b/janeys-pension-plan/janeys-pension-projections.xlsx
@@ -125,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -140,7 +140,6 @@
     <xf numFmtId="165" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -819,12 +818,12 @@
           <t>Full new State Pension per year (£)</t>
         </is>
       </c>
-      <c r="B29" s="11" t="n">
-        <v>11973</v>
+      <c r="B29" s="7" t="n">
+        <v>12500</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>2025/26 full rate ≈ £11,973. Verify current figure at gov.uk.</t>
+          <t>Janey's forecast: £12,500/yr with FULL payments (confirmed) — no NI gaps to fill.</t>
         </is>
       </c>
     </row>
@@ -834,12 +833,12 @@
           <t>% of full State Pension Janey will qualify for</t>
         </is>
       </c>
-      <c r="B30" s="14" t="n">
+      <c r="B30" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>UNKNOWN — get a forecast at gov.uk/check-state-pension. As a homemaker there may be NI gaps; filling them is often the best-value action of all.</t>
+          <t>100% — full payments confirmed.</t>
         </is>
       </c>
     </row>
@@ -851,7 +850,7 @@
       </c>
       <c r="B31" s="10">
         <f>B29*B30</f>
-        <v>11973</v>
+        <v>12500</v>
       </c>
     </row>
     <row r="32">
@@ -1158,333 +1157,333 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>Age</t>
         </is>
       </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>Opening balance</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
+      <c r="D4" s="14" t="inlineStr">
         <is>
           <t>Contribution (gross)</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
+      <c r="E4" s="14" t="inlineStr">
         <is>
           <t>Growth</t>
         </is>
       </c>
-      <c r="F4" s="15" t="inlineStr">
+      <c r="F4" s="14" t="inlineStr">
         <is>
           <t>Closing balance</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="n">
+      <c r="A5" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="16">
+      <c r="B5" s="15">
         <f>Inputs!B5+1</f>
         <v>54</v>
       </c>
-      <c r="C5" s="17">
+      <c r="C5" s="16">
         <f>Inputs!B15</f>
         <v>0</v>
       </c>
-      <c r="D5" s="17">
+      <c r="D5" s="16">
         <f>Inputs!B14</f>
         <v>3600</v>
       </c>
-      <c r="E5" s="18">
+      <c r="E5" s="17">
         <f>(C5+D5)*Inputs!B23</f>
         <v>162</v>
       </c>
-      <c r="F5" s="18">
+      <c r="F5" s="17">
         <f>C5+D5+E5</f>
         <v>3762</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="n">
+      <c r="A6" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="16">
+      <c r="B6" s="15">
         <f>B5+1</f>
         <v>55</v>
       </c>
-      <c r="C6" s="18">
+      <c r="C6" s="17">
         <f>F5</f>
         <v>3762</v>
       </c>
-      <c r="D6" s="17">
+      <c r="D6" s="16">
         <f>Inputs!B14</f>
         <v>3600</v>
       </c>
-      <c r="E6" s="18">
+      <c r="E6" s="17">
         <f>(C6+D6)*Inputs!B23</f>
         <v>331.29</v>
       </c>
-      <c r="F6" s="18">
+      <c r="F6" s="17">
         <f>C6+D6+E6</f>
         <v>7693.29</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="n">
+      <c r="A7" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B7" s="15">
         <f>B6+1</f>
         <v>56</v>
       </c>
-      <c r="C7" s="18">
+      <c r="C7" s="17">
         <f>F6</f>
         <v>7693.29</v>
       </c>
-      <c r="D7" s="17">
+      <c r="D7" s="16">
         <f>Inputs!B14</f>
         <v>3600</v>
       </c>
-      <c r="E7" s="18">
+      <c r="E7" s="17">
         <f>(C7+D7)*Inputs!B23</f>
         <v>508.19805</v>
       </c>
-      <c r="F7" s="18">
+      <c r="F7" s="17">
         <f>C7+D7+E7</f>
         <v>11801.48805</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="n">
+      <c r="A8" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="16">
+      <c r="B8" s="15">
         <f>B7+1</f>
         <v>57</v>
       </c>
-      <c r="C8" s="18">
+      <c r="C8" s="17">
         <f>F7</f>
         <v>11801.48805</v>
       </c>
-      <c r="D8" s="17">
+      <c r="D8" s="16">
         <f>Inputs!B14</f>
         <v>3600</v>
       </c>
-      <c r="E8" s="18">
+      <c r="E8" s="17">
         <f>(C8+D8)*Inputs!B23</f>
         <v>693.066962</v>
       </c>
-      <c r="F8" s="18">
+      <c r="F8" s="17">
         <f>C8+D8+E8</f>
         <v>16094.555012</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="n">
+      <c r="A9" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="15">
         <f>B8+1</f>
         <v>58</v>
       </c>
-      <c r="C9" s="18">
+      <c r="C9" s="17">
         <f>F8</f>
         <v>16094.555012</v>
       </c>
-      <c r="D9" s="17">
+      <c r="D9" s="16">
         <f>Inputs!B14</f>
         <v>3600</v>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="17">
         <f>(C9+D9)*Inputs!B23</f>
         <v>886.254976</v>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="17">
         <f>C9+D9+E9</f>
         <v>20580.809988</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="n">
+      <c r="A10" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="16">
+      <c r="B10" s="15">
         <f>B9+1</f>
         <v>59</v>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="17">
         <f>F9</f>
         <v>20580.809988</v>
       </c>
-      <c r="D10" s="17">
+      <c r="D10" s="16">
         <f>Inputs!B14</f>
         <v>3600</v>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="17">
         <f>(C10+D10)*Inputs!B23</f>
         <v>1088.136449</v>
       </c>
-      <c r="F10" s="18">
+      <c r="F10" s="17">
         <f>C10+D10+E10</f>
         <v>25268.946437</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="n">
+      <c r="A11" s="15" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="16">
+      <c r="B11" s="15">
         <f>B10+1</f>
         <v>60</v>
       </c>
-      <c r="C11" s="18">
+      <c r="C11" s="17">
         <f>F10</f>
         <v>25268.946437</v>
       </c>
-      <c r="D11" s="17">
+      <c r="D11" s="16">
         <f>Inputs!B14</f>
         <v>3600</v>
       </c>
-      <c r="E11" s="18">
+      <c r="E11" s="17">
         <f>(C11+D11)*Inputs!B23</f>
         <v>1299.10259</v>
       </c>
-      <c r="F11" s="18">
+      <c r="F11" s="17">
         <f>C11+D11+E11</f>
         <v>30168.049027</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="n">
+      <c r="A12" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="16">
+      <c r="B12" s="15">
         <f>B11+1</f>
         <v>61</v>
       </c>
-      <c r="C12" s="18">
+      <c r="C12" s="17">
         <f>F11</f>
         <v>30168.049027</v>
       </c>
-      <c r="D12" s="17">
+      <c r="D12" s="16">
         <f>Inputs!B14</f>
         <v>3600</v>
       </c>
-      <c r="E12" s="18">
+      <c r="E12" s="17">
         <f>(C12+D12)*Inputs!B23</f>
         <v>1519.562206</v>
       </c>
-      <c r="F12" s="18">
+      <c r="F12" s="17">
         <f>C12+D12+E12</f>
         <v>35287.611233</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="n">
+      <c r="A13" s="15" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="16">
+      <c r="B13" s="15">
         <f>B12+1</f>
         <v>62</v>
       </c>
-      <c r="C13" s="18">
+      <c r="C13" s="17">
         <f>F12</f>
         <v>35287.611233</v>
       </c>
-      <c r="D13" s="17">
+      <c r="D13" s="16">
         <f>Inputs!B14</f>
         <v>3600</v>
       </c>
-      <c r="E13" s="18">
+      <c r="E13" s="17">
         <f>(C13+D13)*Inputs!B23</f>
         <v>1749.942505</v>
       </c>
-      <c r="F13" s="18">
+      <c r="F13" s="17">
         <f>C13+D13+E13</f>
         <v>40637.553739</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="n">
+      <c r="A14" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="16">
+      <c r="B14" s="15">
         <f>B13+1</f>
         <v>63</v>
       </c>
-      <c r="C14" s="18">
+      <c r="C14" s="17">
         <f>F13</f>
         <v>40637.553739</v>
       </c>
-      <c r="D14" s="17">
+      <c r="D14" s="16">
         <f>Inputs!B14</f>
         <v>3600</v>
       </c>
-      <c r="E14" s="18">
+      <c r="E14" s="17">
         <f>(C14+D14)*Inputs!B23</f>
         <v>1990.689918</v>
       </c>
-      <c r="F14" s="18">
+      <c r="F14" s="17">
         <f>C14+D14+E14</f>
         <v>46228.243657</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="n">
+      <c r="A15" s="15" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="16">
+      <c r="B15" s="15">
         <f>B14+1</f>
         <v>64</v>
       </c>
-      <c r="C15" s="18">
+      <c r="C15" s="17">
         <f>F14</f>
         <v>46228.243657</v>
       </c>
-      <c r="D15" s="17">
+      <c r="D15" s="16">
         <f>Inputs!B14</f>
         <v>3600</v>
       </c>
-      <c r="E15" s="18">
+      <c r="E15" s="17">
         <f>(C15+D15)*Inputs!B23</f>
         <v>2242.270965</v>
       </c>
-      <c r="F15" s="18">
+      <c r="F15" s="17">
         <f>C15+D15+E15</f>
         <v>52070.514621</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="n">
+      <c r="A16" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="16">
+      <c r="B16" s="15">
         <f>B15+1</f>
         <v>65</v>
       </c>
-      <c r="C16" s="18">
+      <c r="C16" s="17">
         <f>F15</f>
         <v>52070.514621</v>
       </c>
-      <c r="D16" s="17">
+      <c r="D16" s="16">
         <f>Inputs!B14</f>
         <v>3600</v>
       </c>
-      <c r="E16" s="18">
+      <c r="E16" s="17">
         <f>(C16+D16)*Inputs!B23</f>
         <v>2505.173158</v>
       </c>
-      <c r="F16" s="18">
+      <c r="F16" s="17">
         <f>C16+D16+E16</f>
         <v>58175.687779</v>
       </c>
@@ -1524,7 +1523,7 @@
           <t>Pot at retirement (age 65)</t>
         </is>
       </c>
-      <c r="F21" s="19">
+      <c r="F21" s="18">
         <f>F16</f>
         <v>58175.687779</v>
       </c>
@@ -1572,63 +1571,63 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>Scenario</t>
         </is>
       </c>
-      <c r="B5" s="20" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>Net growth</t>
         </is>
       </c>
-      <c r="C5" s="20" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>Pot at 65</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Cautious</t>
         </is>
       </c>
-      <c r="B6" s="21">
+      <c r="B6" s="20">
         <f>Inputs!B22</f>
         <v>0.025</v>
       </c>
-      <c r="C6" s="18">
+      <c r="C6" s="17">
         <f>FV(Inputs!B22,Inputs!B8,-Inputs!B14,-Inputs!B15,1)</f>
         <v>50905.590459</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>Central</t>
         </is>
       </c>
-      <c r="B7" s="21">
+      <c r="B7" s="20">
         <f>Inputs!B23</f>
         <v>0.045</v>
       </c>
-      <c r="C7" s="18">
+      <c r="C7" s="17">
         <f>FV(Inputs!B23,Inputs!B8,-Inputs!B14,-Inputs!B15,1)</f>
         <v>58175.687779</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>Optimistic</t>
         </is>
       </c>
-      <c r="B8" s="21">
+      <c r="B8" s="20">
         <f>Inputs!B24</f>
         <v>0.065</v>
       </c>
-      <c r="C8" s="18">
+      <c r="C8" s="17">
         <f>FV(Inputs!B24,Inputs!B8,-Inputs!B14,-Inputs!B15,1)</f>
         <v>66599.30754</v>
       </c>
@@ -1707,79 +1706,79 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="15" t="inlineStr">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>Component</t>
         </is>
       </c>
-      <c r="B18" s="15" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>Age 65–66 (bridge)</t>
         </is>
       </c>
-      <c r="C18" s="15" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>Age 67+ (with SP)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>Private pension (drawdown)</t>
         </is>
       </c>
-      <c r="B19" s="18">
+      <c r="B19" s="17">
         <f>B14</f>
         <v>2327.027511</v>
       </c>
-      <c r="C19" s="18">
+      <c r="C19" s="17">
         <f>B14</f>
         <v>2327.027511</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>Deferred DB (school) pension</t>
         </is>
       </c>
-      <c r="B20" s="17">
+      <c r="B20" s="16">
         <f>Inputs!B32</f>
         <v>6981.65</v>
       </c>
-      <c r="C20" s="17">
+      <c r="C20" s="16">
         <f>Inputs!B32</f>
         <v>6981.65</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>State Pension</t>
         </is>
       </c>
-      <c r="B21" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="C21" s="17">
+      <c r="B21" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="16">
         <f>Inputs!B31</f>
-        <v>11973</v>
+        <v>12500</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="22" t="inlineStr">
+      <c r="A22" s="21" t="inlineStr">
         <is>
           <t>Total annual income</t>
         </is>
       </c>
-      <c r="B22" s="23">
+      <c r="B22" s="22">
         <f>SUM(B19:B21)</f>
         <v>9308.677511</v>
       </c>
-      <c r="C22" s="23">
+      <c r="C22" s="22">
         <f>SUM(C19:C21)</f>
-        <v>21281.677511</v>
+        <v>21808.677511</v>
       </c>
     </row>
     <row r="24">
@@ -1799,7 +1798,7 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>1. Get Janey's State Pension forecast (gov.uk/check-state-pension) — fill NI gaps if any.</t>
+          <t>1. Janey's State Pension confirmed at £12,500/yr, full payments — no NI gaps to fill.</t>
         </is>
       </c>
     </row>
@@ -1866,101 +1865,101 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>Component</t>
         </is>
       </c>
-      <c r="B5" s="20" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>Janey</t>
         </is>
       </c>
-      <c r="C5" s="20" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>Michael</t>
         </is>
       </c>
-      <c r="D5" s="20" t="inlineStr">
+      <c r="D5" s="19" t="inlineStr">
         <is>
           <t>Household</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Private pension (drawdown ~4%)</t>
         </is>
       </c>
-      <c r="B6" s="17">
+      <c r="B6" s="16">
         <f>'Retirement income'!B14</f>
         <v>2327.027511</v>
       </c>
-      <c r="C6" s="17">
+      <c r="C6" s="16">
         <f>Inputs!B43</f>
         <v>25365.606094</v>
       </c>
-      <c r="D6" s="18">
+      <c r="D6" s="17">
         <f>B6+C6</f>
         <v>27692.633606</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>DB / service pension (Teachers' · RAF)</t>
         </is>
       </c>
-      <c r="B7" s="17">
+      <c r="B7" s="16">
         <f>Inputs!B32</f>
         <v>6981.65</v>
       </c>
-      <c r="C7" s="17">
+      <c r="C7" s="16">
         <f>Inputs!B53</f>
         <v>5340</v>
       </c>
-      <c r="D7" s="18">
+      <c r="D7" s="17">
         <f>B7+C7</f>
         <v>12321.65</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>State Pension</t>
         </is>
       </c>
-      <c r="B8" s="17">
+      <c r="B8" s="16">
         <f>Inputs!B31</f>
-        <v>11973</v>
-      </c>
-      <c r="C8" s="17">
+        <v>12500</v>
+      </c>
+      <c r="C8" s="16">
         <f>Inputs!B39</f>
         <v>12532</v>
       </c>
-      <c r="D8" s="18">
+      <c r="D8" s="17">
         <f>B8+C8</f>
-        <v>24505</v>
+        <v>25032</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>Total annual income</t>
         </is>
       </c>
-      <c r="B9" s="23">
+      <c r="B9" s="22">
         <f>SUM(B6:B8)</f>
-        <v>21281.677511</v>
-      </c>
-      <c r="C9" s="23">
+        <v>21808.677511</v>
+      </c>
+      <c r="C9" s="22">
         <f>SUM(C6:C8)</f>
         <v>43237.606094</v>
       </c>
-      <c r="D9" s="23">
+      <c r="D9" s="22">
         <f>SUM(D6:D8)</f>
-        <v>64519.283606</v>
+        <v>65046.283606</v>
       </c>
     </row>
     <row r="10">
@@ -1971,7 +1970,7 @@
       </c>
       <c r="D10" s="8">
         <f>D9/12</f>
-        <v>5376.606967</v>
+        <v>5420.523634</v>
       </c>
     </row>
     <row r="12">
@@ -1982,62 +1981,62 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="B13" s="15" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
         <is>
           <t>Couple / yr</t>
         </is>
       </c>
-      <c r="C13" s="15" t="inlineStr">
+      <c r="C13" s="14" t="inlineStr">
         <is>
           <t>Household vs benchmark</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Minimum</t>
         </is>
       </c>
-      <c r="B14" s="24" t="n">
+      <c r="B14" s="23" t="n">
         <v>22400</v>
       </c>
-      <c r="C14" s="25">
+      <c r="C14" s="24">
         <f>D9-B14</f>
-        <v>42119.283606</v>
+        <v>42646.283606</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="B15" s="24" t="n">
+      <c r="B15" s="23" t="n">
         <v>43100</v>
       </c>
-      <c r="C15" s="25">
+      <c r="C15" s="24">
         <f>D9-B15</f>
-        <v>21419.283606</v>
+        <v>21946.283606</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>Comfortable</t>
         </is>
       </c>
-      <c r="B16" s="24" t="n">
+      <c r="B16" s="23" t="n">
         <v>59000</v>
       </c>
-      <c r="C16" s="25">
+      <c r="C16" s="24">
         <f>D9-B16</f>
-        <v>5519.283606</v>
+        <v>6046.283606</v>
       </c>
     </row>
     <row r="17">
@@ -2132,964 +2131,964 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>Mike</t>
         </is>
       </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>Jane</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
+      <c r="D4" s="14" t="inlineStr">
         <is>
           <t>Mike RAF</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
+      <c r="E4" s="14" t="inlineStr">
         <is>
           <t>Mike pot</t>
         </is>
       </c>
-      <c r="F4" s="15" t="inlineStr">
+      <c r="F4" s="14" t="inlineStr">
         <is>
           <t>Mike State</t>
         </is>
       </c>
-      <c r="G4" s="15" t="inlineStr">
+      <c r="G4" s="14" t="inlineStr">
         <is>
           <t>Jane Tchr</t>
         </is>
       </c>
-      <c r="H4" s="15" t="inlineStr">
+      <c r="H4" s="14" t="inlineStr">
         <is>
           <t>Jane pot</t>
         </is>
       </c>
-      <c r="I4" s="15" t="inlineStr">
+      <c r="I4" s="14" t="inlineStr">
         <is>
           <t>Jane State</t>
         </is>
       </c>
-      <c r="J4" s="15" t="inlineStr">
+      <c r="J4" s="14" t="inlineStr">
         <is>
           <t>Household /yr</t>
         </is>
       </c>
-      <c r="K4" s="15" t="inlineStr">
+      <c r="K4" s="14" t="inlineStr">
         <is>
           <t>Lump sums</t>
         </is>
       </c>
-      <c r="L4" s="15" t="inlineStr">
+      <c r="L4" s="14" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="n">
+      <c r="A5" s="15" t="n">
         <v>2026</v>
       </c>
-      <c r="B5" s="16">
+      <c r="B5" s="15">
         <f>A5-1969</f>
         <v>57</v>
       </c>
-      <c r="C5" s="16">
+      <c r="C5" s="15">
         <f>A5-1972</f>
         <v>54</v>
       </c>
-      <c r="D5" s="18">
+      <c r="D5" s="17">
         <f>IF(B5&gt;=60,Inputs!B53,0)</f>
         <v>0</v>
       </c>
-      <c r="E5" s="18">
+      <c r="E5" s="17">
         <f>IF(B5&gt;=Inputs!B36,Inputs!B43,0)</f>
         <v>0</v>
       </c>
-      <c r="F5" s="18">
+      <c r="F5" s="17">
         <f>IF(B5&gt;=67,Inputs!B39,0)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="18">
+      <c r="G5" s="17">
         <f>IF(C5&gt;=60,Inputs!B32,0)</f>
         <v>0</v>
       </c>
-      <c r="H5" s="18">
+      <c r="H5" s="17">
         <f>IF(C5&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
         <v>0</v>
       </c>
-      <c r="I5" s="18">
+      <c r="I5" s="17">
         <f>IF(C5&gt;=67,Inputs!B31,0)</f>
         <v>0</v>
       </c>
-      <c r="J5" s="23">
+      <c r="J5" s="22">
         <f>SUM(D5:I5)</f>
         <v>0</v>
       </c>
-      <c r="K5" s="18">
+      <c r="K5" s="17">
         <f>IF(B5=60,Inputs!B54,0)+IF(C5=60,Inputs!B47,0)</f>
         <v>0</v>
       </c>
-      <c r="L5" s="26" t="n"/>
+      <c r="L5" s="25" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="n">
+      <c r="A6" s="15" t="n">
         <v>2027</v>
       </c>
-      <c r="B6" s="16">
+      <c r="B6" s="15">
         <f>A6-1969</f>
         <v>58</v>
       </c>
-      <c r="C6" s="16">
+      <c r="C6" s="15">
         <f>A6-1972</f>
         <v>55</v>
       </c>
-      <c r="D6" s="18">
+      <c r="D6" s="17">
         <f>IF(B6&gt;=60,Inputs!B53,0)</f>
         <v>0</v>
       </c>
-      <c r="E6" s="18">
+      <c r="E6" s="17">
         <f>IF(B6&gt;=Inputs!B36,Inputs!B43,0)</f>
         <v>0</v>
       </c>
-      <c r="F6" s="18">
+      <c r="F6" s="17">
         <f>IF(B6&gt;=67,Inputs!B39,0)</f>
         <v>0</v>
       </c>
-      <c r="G6" s="18">
+      <c r="G6" s="17">
         <f>IF(C6&gt;=60,Inputs!B32,0)</f>
         <v>0</v>
       </c>
-      <c r="H6" s="18">
+      <c r="H6" s="17">
         <f>IF(C6&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
         <v>0</v>
       </c>
-      <c r="I6" s="18">
+      <c r="I6" s="17">
         <f>IF(C6&gt;=67,Inputs!B31,0)</f>
         <v>0</v>
       </c>
-      <c r="J6" s="23">
+      <c r="J6" s="22">
         <f>SUM(D6:I6)</f>
         <v>0</v>
       </c>
-      <c r="K6" s="18">
+      <c r="K6" s="17">
         <f>IF(B6=60,Inputs!B54,0)+IF(C6=60,Inputs!B47,0)</f>
         <v>0</v>
       </c>
-      <c r="L6" s="26" t="n"/>
+      <c r="L6" s="25" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="n">
+      <c r="A7" s="15" t="n">
         <v>2028</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B7" s="15">
         <f>A7-1969</f>
         <v>59</v>
       </c>
-      <c r="C7" s="16">
+      <c r="C7" s="15">
         <f>A7-1972</f>
         <v>56</v>
       </c>
-      <c r="D7" s="18">
+      <c r="D7" s="17">
         <f>IF(B7&gt;=60,Inputs!B53,0)</f>
         <v>0</v>
       </c>
-      <c r="E7" s="18">
+      <c r="E7" s="17">
         <f>IF(B7&gt;=Inputs!B36,Inputs!B43,0)</f>
         <v>0</v>
       </c>
-      <c r="F7" s="18">
+      <c r="F7" s="17">
         <f>IF(B7&gt;=67,Inputs!B39,0)</f>
         <v>0</v>
       </c>
-      <c r="G7" s="18">
+      <c r="G7" s="17">
         <f>IF(C7&gt;=60,Inputs!B32,0)</f>
         <v>0</v>
       </c>
-      <c r="H7" s="18">
+      <c r="H7" s="17">
         <f>IF(C7&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
         <v>0</v>
       </c>
-      <c r="I7" s="18">
+      <c r="I7" s="17">
         <f>IF(C7&gt;=67,Inputs!B31,0)</f>
         <v>0</v>
       </c>
-      <c r="J7" s="23">
+      <c r="J7" s="22">
         <f>SUM(D7:I7)</f>
         <v>0</v>
       </c>
-      <c r="K7" s="18">
+      <c r="K7" s="17">
         <f>IF(B7=60,Inputs!B54,0)+IF(C7=60,Inputs!B47,0)</f>
         <v>0</v>
       </c>
-      <c r="L7" s="26" t="n"/>
+      <c r="L7" s="25" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="n">
+      <c r="A8" s="15" t="n">
         <v>2029</v>
       </c>
-      <c r="B8" s="16">
+      <c r="B8" s="15">
         <f>A8-1969</f>
         <v>60</v>
       </c>
-      <c r="C8" s="16">
+      <c r="C8" s="15">
         <f>A8-1972</f>
         <v>57</v>
       </c>
-      <c r="D8" s="18">
+      <c r="D8" s="17">
         <f>IF(B8&gt;=60,Inputs!B53,0)</f>
         <v>5340</v>
       </c>
-      <c r="E8" s="18">
+      <c r="E8" s="17">
         <f>IF(B8&gt;=Inputs!B36,Inputs!B43,0)</f>
         <v>0</v>
       </c>
-      <c r="F8" s="18">
+      <c r="F8" s="17">
         <f>IF(B8&gt;=67,Inputs!B39,0)</f>
         <v>0</v>
       </c>
-      <c r="G8" s="18">
+      <c r="G8" s="17">
         <f>IF(C8&gt;=60,Inputs!B32,0)</f>
         <v>0</v>
       </c>
-      <c r="H8" s="18">
+      <c r="H8" s="17">
         <f>IF(C8&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
         <v>0</v>
       </c>
-      <c r="I8" s="18">
+      <c r="I8" s="17">
         <f>IF(C8&gt;=67,Inputs!B31,0)</f>
         <v>0</v>
       </c>
-      <c r="J8" s="23">
+      <c r="J8" s="22">
         <f>SUM(D8:I8)</f>
         <v>5340</v>
       </c>
-      <c r="K8" s="18">
+      <c r="K8" s="17">
         <f>IF(B8=60,Inputs!B54,0)+IF(C8=60,Inputs!B47,0)</f>
         <v>16020</v>
       </c>
-      <c r="L8" s="27" t="inlineStr">
+      <c r="L8" s="26" t="inlineStr">
         <is>
           <t>Mike 60 → RAF pension + lump sum</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="n">
+      <c r="A9" s="15" t="n">
         <v>2030</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="15">
         <f>A9-1969</f>
         <v>61</v>
       </c>
-      <c r="C9" s="16">
+      <c r="C9" s="15">
         <f>A9-1972</f>
         <v>58</v>
       </c>
-      <c r="D9" s="18">
+      <c r="D9" s="17">
         <f>IF(B9&gt;=60,Inputs!B53,0)</f>
         <v>5340</v>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="17">
         <f>IF(B9&gt;=Inputs!B36,Inputs!B43,0)</f>
         <v>0</v>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="17">
         <f>IF(B9&gt;=67,Inputs!B39,0)</f>
         <v>0</v>
       </c>
-      <c r="G9" s="18">
+      <c r="G9" s="17">
         <f>IF(C9&gt;=60,Inputs!B32,0)</f>
         <v>0</v>
       </c>
-      <c r="H9" s="18">
+      <c r="H9" s="17">
         <f>IF(C9&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
         <v>0</v>
       </c>
-      <c r="I9" s="18">
+      <c r="I9" s="17">
         <f>IF(C9&gt;=67,Inputs!B31,0)</f>
         <v>0</v>
       </c>
-      <c r="J9" s="23">
+      <c r="J9" s="22">
         <f>SUM(D9:I9)</f>
         <v>5340</v>
       </c>
-      <c r="K9" s="18">
+      <c r="K9" s="17">
         <f>IF(B9=60,Inputs!B54,0)+IF(C9=60,Inputs!B47,0)</f>
         <v>0</v>
       </c>
-      <c r="L9" s="26" t="n"/>
+      <c r="L9" s="25" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="n">
+      <c r="A10" s="15" t="n">
         <v>2031</v>
       </c>
-      <c r="B10" s="16">
+      <c r="B10" s="15">
         <f>A10-1969</f>
         <v>62</v>
       </c>
-      <c r="C10" s="16">
+      <c r="C10" s="15">
         <f>A10-1972</f>
         <v>59</v>
       </c>
-      <c r="D10" s="18">
+      <c r="D10" s="17">
         <f>IF(B10&gt;=60,Inputs!B53,0)</f>
         <v>5340</v>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="17">
         <f>IF(B10&gt;=Inputs!B36,Inputs!B43,0)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="18">
+      <c r="F10" s="17">
         <f>IF(B10&gt;=67,Inputs!B39,0)</f>
         <v>0</v>
       </c>
-      <c r="G10" s="18">
+      <c r="G10" s="17">
         <f>IF(C10&gt;=60,Inputs!B32,0)</f>
         <v>0</v>
       </c>
-      <c r="H10" s="18">
+      <c r="H10" s="17">
         <f>IF(C10&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
         <v>0</v>
       </c>
-      <c r="I10" s="18">
+      <c r="I10" s="17">
         <f>IF(C10&gt;=67,Inputs!B31,0)</f>
         <v>0</v>
       </c>
-      <c r="J10" s="23">
+      <c r="J10" s="22">
         <f>SUM(D10:I10)</f>
         <v>5340</v>
       </c>
-      <c r="K10" s="18">
+      <c r="K10" s="17">
         <f>IF(B10=60,Inputs!B54,0)+IF(C10=60,Inputs!B47,0)</f>
         <v>0</v>
       </c>
-      <c r="L10" s="26" t="n"/>
+      <c r="L10" s="25" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="n">
+      <c r="A11" s="15" t="n">
         <v>2032</v>
       </c>
-      <c r="B11" s="16">
+      <c r="B11" s="15">
         <f>A11-1969</f>
         <v>63</v>
       </c>
-      <c r="C11" s="16">
+      <c r="C11" s="15">
         <f>A11-1972</f>
         <v>60</v>
       </c>
-      <c r="D11" s="18">
+      <c r="D11" s="17">
         <f>IF(B11&gt;=60,Inputs!B53,0)</f>
         <v>5340</v>
       </c>
-      <c r="E11" s="18">
+      <c r="E11" s="17">
         <f>IF(B11&gt;=Inputs!B36,Inputs!B43,0)</f>
         <v>0</v>
       </c>
-      <c r="F11" s="18">
+      <c r="F11" s="17">
         <f>IF(B11&gt;=67,Inputs!B39,0)</f>
         <v>0</v>
       </c>
-      <c r="G11" s="18">
+      <c r="G11" s="17">
         <f>IF(C11&gt;=60,Inputs!B32,0)</f>
         <v>6981.65</v>
       </c>
-      <c r="H11" s="18">
+      <c r="H11" s="17">
         <f>IF(C11&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
         <v>0</v>
       </c>
-      <c r="I11" s="18">
+      <c r="I11" s="17">
         <f>IF(C11&gt;=67,Inputs!B31,0)</f>
         <v>0</v>
       </c>
-      <c r="J11" s="23">
+      <c r="J11" s="22">
         <f>SUM(D11:I11)</f>
         <v>12321.65</v>
       </c>
-      <c r="K11" s="18">
+      <c r="K11" s="17">
         <f>IF(B11=60,Inputs!B54,0)+IF(C11=60,Inputs!B47,0)</f>
         <v>20944.98</v>
       </c>
-      <c r="L11" s="27" t="inlineStr">
+      <c r="L11" s="26" t="inlineStr">
         <is>
           <t>Jane 60 → Teachers' pension + lump sum</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="n">
+      <c r="A12" s="15" t="n">
         <v>2033</v>
       </c>
-      <c r="B12" s="16">
+      <c r="B12" s="15">
         <f>A12-1969</f>
         <v>64</v>
       </c>
-      <c r="C12" s="16">
+      <c r="C12" s="15">
         <f>A12-1972</f>
         <v>61</v>
       </c>
-      <c r="D12" s="18">
+      <c r="D12" s="17">
         <f>IF(B12&gt;=60,Inputs!B53,0)</f>
         <v>5340</v>
       </c>
-      <c r="E12" s="18">
+      <c r="E12" s="17">
         <f>IF(B12&gt;=Inputs!B36,Inputs!B43,0)</f>
         <v>0</v>
       </c>
-      <c r="F12" s="18">
+      <c r="F12" s="17">
         <f>IF(B12&gt;=67,Inputs!B39,0)</f>
         <v>0</v>
       </c>
-      <c r="G12" s="18">
+      <c r="G12" s="17">
         <f>IF(C12&gt;=60,Inputs!B32,0)</f>
         <v>6981.65</v>
       </c>
-      <c r="H12" s="18">
+      <c r="H12" s="17">
         <f>IF(C12&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
         <v>0</v>
       </c>
-      <c r="I12" s="18">
+      <c r="I12" s="17">
         <f>IF(C12&gt;=67,Inputs!B31,0)</f>
         <v>0</v>
       </c>
-      <c r="J12" s="23">
+      <c r="J12" s="22">
         <f>SUM(D12:I12)</f>
         <v>12321.65</v>
       </c>
-      <c r="K12" s="18">
+      <c r="K12" s="17">
         <f>IF(B12=60,Inputs!B54,0)+IF(C12=60,Inputs!B47,0)</f>
         <v>0</v>
       </c>
-      <c r="L12" s="26" t="n"/>
+      <c r="L12" s="25" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="n">
+      <c r="A13" s="15" t="n">
         <v>2034</v>
       </c>
-      <c r="B13" s="16">
+      <c r="B13" s="15">
         <f>A13-1969</f>
         <v>65</v>
       </c>
-      <c r="C13" s="16">
+      <c r="C13" s="15">
         <f>A13-1972</f>
         <v>62</v>
       </c>
-      <c r="D13" s="18">
+      <c r="D13" s="17">
         <f>IF(B13&gt;=60,Inputs!B53,0)</f>
         <v>5340</v>
       </c>
-      <c r="E13" s="18">
+      <c r="E13" s="17">
         <f>IF(B13&gt;=Inputs!B36,Inputs!B43,0)</f>
         <v>25365.606094</v>
       </c>
-      <c r="F13" s="18">
+      <c r="F13" s="17">
         <f>IF(B13&gt;=67,Inputs!B39,0)</f>
         <v>0</v>
       </c>
-      <c r="G13" s="18">
+      <c r="G13" s="17">
         <f>IF(C13&gt;=60,Inputs!B32,0)</f>
         <v>6981.65</v>
       </c>
-      <c r="H13" s="18">
+      <c r="H13" s="17">
         <f>IF(C13&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
         <v>0</v>
       </c>
-      <c r="I13" s="18">
+      <c r="I13" s="17">
         <f>IF(C13&gt;=67,Inputs!B31,0)</f>
         <v>0</v>
       </c>
-      <c r="J13" s="23">
+      <c r="J13" s="22">
         <f>SUM(D13:I13)</f>
         <v>37687.256094</v>
       </c>
-      <c r="K13" s="18">
+      <c r="K13" s="17">
         <f>IF(B13=60,Inputs!B54,0)+IF(C13=60,Inputs!B47,0)</f>
         <v>0</v>
       </c>
-      <c r="L13" s="27" t="inlineStr">
+      <c r="L13" s="26" t="inlineStr">
         <is>
           <t>Mike 65 → retires, draws DC pot</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="n">
+      <c r="A14" s="15" t="n">
         <v>2035</v>
       </c>
-      <c r="B14" s="16">
+      <c r="B14" s="15">
         <f>A14-1969</f>
         <v>66</v>
       </c>
-      <c r="C14" s="16">
+      <c r="C14" s="15">
         <f>A14-1972</f>
         <v>63</v>
       </c>
-      <c r="D14" s="18">
+      <c r="D14" s="17">
         <f>IF(B14&gt;=60,Inputs!B53,0)</f>
         <v>5340</v>
       </c>
-      <c r="E14" s="18">
+      <c r="E14" s="17">
         <f>IF(B14&gt;=Inputs!B36,Inputs!B43,0)</f>
         <v>25365.606094</v>
       </c>
-      <c r="F14" s="18">
+      <c r="F14" s="17">
         <f>IF(B14&gt;=67,Inputs!B39,0)</f>
         <v>0</v>
       </c>
-      <c r="G14" s="18">
+      <c r="G14" s="17">
         <f>IF(C14&gt;=60,Inputs!B32,0)</f>
         <v>6981.65</v>
       </c>
-      <c r="H14" s="18">
+      <c r="H14" s="17">
         <f>IF(C14&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
         <v>0</v>
       </c>
-      <c r="I14" s="18">
+      <c r="I14" s="17">
         <f>IF(C14&gt;=67,Inputs!B31,0)</f>
         <v>0</v>
       </c>
-      <c r="J14" s="23">
+      <c r="J14" s="22">
         <f>SUM(D14:I14)</f>
         <v>37687.256094</v>
       </c>
-      <c r="K14" s="18">
+      <c r="K14" s="17">
         <f>IF(B14=60,Inputs!B54,0)+IF(C14=60,Inputs!B47,0)</f>
         <v>0</v>
       </c>
-      <c r="L14" s="26" t="n"/>
+      <c r="L14" s="25" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="n">
+      <c r="A15" s="15" t="n">
         <v>2036</v>
       </c>
-      <c r="B15" s="16">
+      <c r="B15" s="15">
         <f>A15-1969</f>
         <v>67</v>
       </c>
-      <c r="C15" s="16">
+      <c r="C15" s="15">
         <f>A15-1972</f>
         <v>64</v>
       </c>
-      <c r="D15" s="18">
+      <c r="D15" s="17">
         <f>IF(B15&gt;=60,Inputs!B53,0)</f>
         <v>5340</v>
       </c>
-      <c r="E15" s="18">
+      <c r="E15" s="17">
         <f>IF(B15&gt;=Inputs!B36,Inputs!B43,0)</f>
         <v>25365.606094</v>
       </c>
-      <c r="F15" s="18">
+      <c r="F15" s="17">
         <f>IF(B15&gt;=67,Inputs!B39,0)</f>
         <v>12532</v>
       </c>
-      <c r="G15" s="18">
+      <c r="G15" s="17">
         <f>IF(C15&gt;=60,Inputs!B32,0)</f>
         <v>6981.65</v>
       </c>
-      <c r="H15" s="18">
+      <c r="H15" s="17">
         <f>IF(C15&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
         <v>0</v>
       </c>
-      <c r="I15" s="18">
+      <c r="I15" s="17">
         <f>IF(C15&gt;=67,Inputs!B31,0)</f>
         <v>0</v>
       </c>
-      <c r="J15" s="23">
+      <c r="J15" s="22">
         <f>SUM(D15:I15)</f>
         <v>50219.256094</v>
       </c>
-      <c r="K15" s="18">
+      <c r="K15" s="17">
         <f>IF(B15=60,Inputs!B54,0)+IF(C15=60,Inputs!B47,0)</f>
         <v>0</v>
       </c>
-      <c r="L15" s="27" t="inlineStr">
+      <c r="L15" s="26" t="inlineStr">
         <is>
           <t>Mike 67 → State Pension starts</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="n">
+      <c r="A16" s="15" t="n">
         <v>2037</v>
       </c>
-      <c r="B16" s="16">
+      <c r="B16" s="15">
         <f>A16-1969</f>
         <v>68</v>
       </c>
-      <c r="C16" s="16">
+      <c r="C16" s="15">
         <f>A16-1972</f>
         <v>65</v>
       </c>
-      <c r="D16" s="18">
+      <c r="D16" s="17">
         <f>IF(B16&gt;=60,Inputs!B53,0)</f>
         <v>5340</v>
       </c>
-      <c r="E16" s="18">
+      <c r="E16" s="17">
         <f>IF(B16&gt;=Inputs!B36,Inputs!B43,0)</f>
         <v>25365.606094</v>
       </c>
-      <c r="F16" s="18">
+      <c r="F16" s="17">
         <f>IF(B16&gt;=67,Inputs!B39,0)</f>
         <v>12532</v>
       </c>
-      <c r="G16" s="18">
+      <c r="G16" s="17">
         <f>IF(C16&gt;=60,Inputs!B32,0)</f>
         <v>6981.65</v>
       </c>
-      <c r="H16" s="18">
+      <c r="H16" s="17">
         <f>IF(C16&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
         <v>2327.027511</v>
       </c>
-      <c r="I16" s="18">
+      <c r="I16" s="17">
         <f>IF(C16&gt;=67,Inputs!B31,0)</f>
         <v>0</v>
       </c>
-      <c r="J16" s="23">
+      <c r="J16" s="22">
         <f>SUM(D16:I16)</f>
         <v>52546.283606</v>
       </c>
-      <c r="K16" s="18">
+      <c r="K16" s="17">
         <f>IF(B16=60,Inputs!B54,0)+IF(C16=60,Inputs!B47,0)</f>
         <v>0</v>
       </c>
-      <c r="L16" s="27" t="inlineStr">
+      <c r="L16" s="26" t="inlineStr">
         <is>
           <t>Jane 65 → retires, draws DC pot</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="n">
+      <c r="A17" s="15" t="n">
         <v>2038</v>
       </c>
-      <c r="B17" s="16">
+      <c r="B17" s="15">
         <f>A17-1969</f>
         <v>69</v>
       </c>
-      <c r="C17" s="16">
+      <c r="C17" s="15">
         <f>A17-1972</f>
         <v>66</v>
       </c>
-      <c r="D17" s="18">
+      <c r="D17" s="17">
         <f>IF(B17&gt;=60,Inputs!B53,0)</f>
         <v>5340</v>
       </c>
-      <c r="E17" s="18">
+      <c r="E17" s="17">
         <f>IF(B17&gt;=Inputs!B36,Inputs!B43,0)</f>
         <v>25365.606094</v>
       </c>
-      <c r="F17" s="18">
+      <c r="F17" s="17">
         <f>IF(B17&gt;=67,Inputs!B39,0)</f>
         <v>12532</v>
       </c>
-      <c r="G17" s="18">
+      <c r="G17" s="17">
         <f>IF(C17&gt;=60,Inputs!B32,0)</f>
         <v>6981.65</v>
       </c>
-      <c r="H17" s="18">
+      <c r="H17" s="17">
         <f>IF(C17&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
         <v>2327.027511</v>
       </c>
-      <c r="I17" s="18">
+      <c r="I17" s="17">
         <f>IF(C17&gt;=67,Inputs!B31,0)</f>
         <v>0</v>
       </c>
-      <c r="J17" s="23">
+      <c r="J17" s="22">
         <f>SUM(D17:I17)</f>
         <v>52546.283606</v>
       </c>
-      <c r="K17" s="18">
+      <c r="K17" s="17">
         <f>IF(B17=60,Inputs!B54,0)+IF(C17=60,Inputs!B47,0)</f>
         <v>0</v>
       </c>
-      <c r="L17" s="26" t="n"/>
+      <c r="L17" s="25" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="n">
+      <c r="A18" s="15" t="n">
         <v>2039</v>
       </c>
-      <c r="B18" s="16">
+      <c r="B18" s="15">
         <f>A18-1969</f>
         <v>70</v>
       </c>
-      <c r="C18" s="16">
+      <c r="C18" s="15">
         <f>A18-1972</f>
         <v>67</v>
       </c>
-      <c r="D18" s="18">
+      <c r="D18" s="17">
         <f>IF(B18&gt;=60,Inputs!B53,0)</f>
         <v>5340</v>
       </c>
-      <c r="E18" s="18">
+      <c r="E18" s="17">
         <f>IF(B18&gt;=Inputs!B36,Inputs!B43,0)</f>
         <v>25365.606094</v>
       </c>
-      <c r="F18" s="18">
+      <c r="F18" s="17">
         <f>IF(B18&gt;=67,Inputs!B39,0)</f>
         <v>12532</v>
       </c>
-      <c r="G18" s="18">
+      <c r="G18" s="17">
         <f>IF(C18&gt;=60,Inputs!B32,0)</f>
         <v>6981.65</v>
       </c>
-      <c r="H18" s="18">
+      <c r="H18" s="17">
         <f>IF(C18&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
         <v>2327.027511</v>
       </c>
-      <c r="I18" s="18">
+      <c r="I18" s="17">
         <f>IF(C18&gt;=67,Inputs!B31,0)</f>
-        <v>11973</v>
-      </c>
-      <c r="J18" s="23">
+        <v>12500</v>
+      </c>
+      <c r="J18" s="22">
         <f>SUM(D18:I18)</f>
-        <v>64519.283606</v>
-      </c>
-      <c r="K18" s="18">
+        <v>65046.283606</v>
+      </c>
+      <c r="K18" s="17">
         <f>IF(B18=60,Inputs!B54,0)+IF(C18=60,Inputs!B47,0)</f>
         <v>0</v>
       </c>
-      <c r="L18" s="27" t="inlineStr">
+      <c r="L18" s="26" t="inlineStr">
         <is>
           <t>Jane 67 → State Pension starts (all streams on)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="n">
+      <c r="A19" s="15" t="n">
         <v>2040</v>
       </c>
-      <c r="B19" s="16">
+      <c r="B19" s="15">
         <f>A19-1969</f>
         <v>71</v>
       </c>
-      <c r="C19" s="16">
+      <c r="C19" s="15">
         <f>A19-1972</f>
         <v>68</v>
       </c>
-      <c r="D19" s="18">
+      <c r="D19" s="17">
         <f>IF(B19&gt;=60,Inputs!B53,0)</f>
         <v>5340</v>
       </c>
-      <c r="E19" s="18">
+      <c r="E19" s="17">
         <f>IF(B19&gt;=Inputs!B36,Inputs!B43,0)</f>
         <v>25365.606094</v>
       </c>
-      <c r="F19" s="18">
+      <c r="F19" s="17">
         <f>IF(B19&gt;=67,Inputs!B39,0)</f>
         <v>12532</v>
       </c>
-      <c r="G19" s="18">
+      <c r="G19" s="17">
         <f>IF(C19&gt;=60,Inputs!B32,0)</f>
         <v>6981.65</v>
       </c>
-      <c r="H19" s="18">
+      <c r="H19" s="17">
         <f>IF(C19&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
         <v>2327.027511</v>
       </c>
-      <c r="I19" s="18">
+      <c r="I19" s="17">
         <f>IF(C19&gt;=67,Inputs!B31,0)</f>
-        <v>11973</v>
-      </c>
-      <c r="J19" s="23">
+        <v>12500</v>
+      </c>
+      <c r="J19" s="22">
         <f>SUM(D19:I19)</f>
-        <v>64519.283606</v>
-      </c>
-      <c r="K19" s="18">
+        <v>65046.283606</v>
+      </c>
+      <c r="K19" s="17">
         <f>IF(B19=60,Inputs!B54,0)+IF(C19=60,Inputs!B47,0)</f>
         <v>0</v>
       </c>
-      <c r="L19" s="26" t="n"/>
+      <c r="L19" s="25" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="n">
+      <c r="A20" s="15" t="n">
         <v>2041</v>
       </c>
-      <c r="B20" s="16">
+      <c r="B20" s="15">
         <f>A20-1969</f>
         <v>72</v>
       </c>
-      <c r="C20" s="16">
+      <c r="C20" s="15">
         <f>A20-1972</f>
         <v>69</v>
       </c>
-      <c r="D20" s="18">
+      <c r="D20" s="17">
         <f>IF(B20&gt;=60,Inputs!B53,0)</f>
         <v>5340</v>
       </c>
-      <c r="E20" s="18">
+      <c r="E20" s="17">
         <f>IF(B20&gt;=Inputs!B36,Inputs!B43,0)</f>
         <v>25365.606094</v>
       </c>
-      <c r="F20" s="18">
+      <c r="F20" s="17">
         <f>IF(B20&gt;=67,Inputs!B39,0)</f>
         <v>12532</v>
       </c>
-      <c r="G20" s="18">
+      <c r="G20" s="17">
         <f>IF(C20&gt;=60,Inputs!B32,0)</f>
         <v>6981.65</v>
       </c>
-      <c r="H20" s="18">
+      <c r="H20" s="17">
         <f>IF(C20&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
         <v>2327.027511</v>
       </c>
-      <c r="I20" s="18">
+      <c r="I20" s="17">
         <f>IF(C20&gt;=67,Inputs!B31,0)</f>
-        <v>11973</v>
-      </c>
-      <c r="J20" s="23">
+        <v>12500</v>
+      </c>
+      <c r="J20" s="22">
         <f>SUM(D20:I20)</f>
-        <v>64519.283606</v>
-      </c>
-      <c r="K20" s="18">
+        <v>65046.283606</v>
+      </c>
+      <c r="K20" s="17">
         <f>IF(B20=60,Inputs!B54,0)+IF(C20=60,Inputs!B47,0)</f>
         <v>0</v>
       </c>
-      <c r="L20" s="26" t="n"/>
+      <c r="L20" s="25" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="n">
+      <c r="A21" s="15" t="n">
         <v>2042</v>
       </c>
-      <c r="B21" s="16">
+      <c r="B21" s="15">
         <f>A21-1969</f>
         <v>73</v>
       </c>
-      <c r="C21" s="16">
+      <c r="C21" s="15">
         <f>A21-1972</f>
         <v>70</v>
       </c>
-      <c r="D21" s="18">
+      <c r="D21" s="17">
         <f>IF(B21&gt;=60,Inputs!B53,0)</f>
         <v>5340</v>
       </c>
-      <c r="E21" s="18">
+      <c r="E21" s="17">
         <f>IF(B21&gt;=Inputs!B36,Inputs!B43,0)</f>
         <v>25365.606094</v>
       </c>
-      <c r="F21" s="18">
+      <c r="F21" s="17">
         <f>IF(B21&gt;=67,Inputs!B39,0)</f>
         <v>12532</v>
       </c>
-      <c r="G21" s="18">
+      <c r="G21" s="17">
         <f>IF(C21&gt;=60,Inputs!B32,0)</f>
         <v>6981.65</v>
       </c>
-      <c r="H21" s="18">
+      <c r="H21" s="17">
         <f>IF(C21&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
         <v>2327.027511</v>
       </c>
-      <c r="I21" s="18">
+      <c r="I21" s="17">
         <f>IF(C21&gt;=67,Inputs!B31,0)</f>
-        <v>11973</v>
-      </c>
-      <c r="J21" s="23">
+        <v>12500</v>
+      </c>
+      <c r="J21" s="22">
         <f>SUM(D21:I21)</f>
-        <v>64519.283606</v>
-      </c>
-      <c r="K21" s="18">
+        <v>65046.283606</v>
+      </c>
+      <c r="K21" s="17">
         <f>IF(B21=60,Inputs!B54,0)+IF(C21=60,Inputs!B47,0)</f>
         <v>0</v>
       </c>
-      <c r="L21" s="26" t="n"/>
+      <c r="L21" s="25" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="n">
+      <c r="A22" s="15" t="n">
         <v>2043</v>
       </c>
-      <c r="B22" s="16">
+      <c r="B22" s="15">
         <f>A22-1969</f>
         <v>74</v>
       </c>
-      <c r="C22" s="16">
+      <c r="C22" s="15">
         <f>A22-1972</f>
         <v>71</v>
       </c>
-      <c r="D22" s="18">
+      <c r="D22" s="17">
         <f>IF(B22&gt;=60,Inputs!B53,0)</f>
         <v>5340</v>
       </c>
-      <c r="E22" s="18">
+      <c r="E22" s="17">
         <f>IF(B22&gt;=Inputs!B36,Inputs!B43,0)</f>
         <v>25365.606094</v>
       </c>
-      <c r="F22" s="18">
+      <c r="F22" s="17">
         <f>IF(B22&gt;=67,Inputs!B39,0)</f>
         <v>12532</v>
       </c>
-      <c r="G22" s="18">
+      <c r="G22" s="17">
         <f>IF(C22&gt;=60,Inputs!B32,0)</f>
         <v>6981.65</v>
       </c>
-      <c r="H22" s="18">
+      <c r="H22" s="17">
         <f>IF(C22&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
         <v>2327.027511</v>
       </c>
-      <c r="I22" s="18">
+      <c r="I22" s="17">
         <f>IF(C22&gt;=67,Inputs!B31,0)</f>
-        <v>11973</v>
-      </c>
-      <c r="J22" s="23">
+        <v>12500</v>
+      </c>
+      <c r="J22" s="22">
         <f>SUM(D22:I22)</f>
-        <v>64519.283606</v>
-      </c>
-      <c r="K22" s="18">
+        <v>65046.283606</v>
+      </c>
+      <c r="K22" s="17">
         <f>IF(B22=60,Inputs!B54,0)+IF(C22=60,Inputs!B47,0)</f>
         <v>0</v>
       </c>
-      <c r="L22" s="26" t="n"/>
+      <c r="L22" s="25" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="n">
+      <c r="A23" s="15" t="n">
         <v>2044</v>
       </c>
-      <c r="B23" s="16">
+      <c r="B23" s="15">
         <f>A23-1969</f>
         <v>75</v>
       </c>
-      <c r="C23" s="16">
+      <c r="C23" s="15">
         <f>A23-1972</f>
         <v>72</v>
       </c>
-      <c r="D23" s="18">
+      <c r="D23" s="17">
         <f>IF(B23&gt;=60,Inputs!B53,0)</f>
         <v>5340</v>
       </c>
-      <c r="E23" s="18">
+      <c r="E23" s="17">
         <f>IF(B23&gt;=Inputs!B36,Inputs!B43,0)</f>
         <v>25365.606094</v>
       </c>
-      <c r="F23" s="18">
+      <c r="F23" s="17">
         <f>IF(B23&gt;=67,Inputs!B39,0)</f>
         <v>12532</v>
       </c>
-      <c r="G23" s="18">
+      <c r="G23" s="17">
         <f>IF(C23&gt;=60,Inputs!B32,0)</f>
         <v>6981.65</v>
       </c>
-      <c r="H23" s="18">
+      <c r="H23" s="17">
         <f>IF(C23&gt;=Inputs!B6,'Retirement income'!B14,0)</f>
         <v>2327.027511</v>
       </c>
-      <c r="I23" s="18">
+      <c r="I23" s="17">
         <f>IF(C23&gt;=67,Inputs!B31,0)</f>
-        <v>11973</v>
-      </c>
-      <c r="J23" s="23">
+        <v>12500</v>
+      </c>
+      <c r="J23" s="22">
         <f>SUM(D23:I23)</f>
-        <v>64519.283606</v>
-      </c>
-      <c r="K23" s="18">
+        <v>65046.283606</v>
+      </c>
+      <c r="K23" s="17">
         <f>IF(B23=60,Inputs!B54,0)+IF(C23=60,Inputs!B47,0)</f>
         <v>0</v>
       </c>
-      <c r="L23" s="26" t="n"/>
+      <c r="L23" s="25" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3161,231 +3160,231 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
+      <c r="B4" s="19" t="inlineStr">
         <is>
           <t>Retire at 60</t>
         </is>
       </c>
-      <c r="C4" s="20" t="inlineStr">
+      <c r="C4" s="19" t="inlineStr">
         <is>
           <t>Retire at 62</t>
         </is>
       </c>
-      <c r="D4" s="20" t="inlineStr">
+      <c r="D4" s="19" t="inlineStr">
         <is>
           <t>Retire at 65</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>Michael's retirement age</t>
         </is>
       </c>
-      <c r="B5" s="28" t="n">
+      <c r="B5" s="27" t="n">
         <v>60</v>
       </c>
-      <c r="C5" s="28" t="n">
+      <c r="C5" s="27" t="n">
         <v>62</v>
       </c>
-      <c r="D5" s="28" t="n">
+      <c r="D5" s="27" t="n">
         <v>65</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Years of contributions</t>
         </is>
       </c>
-      <c r="B6" s="16">
+      <c r="B6" s="15">
         <f>B5-Inputs!B35</f>
         <v>3</v>
       </c>
-      <c r="C6" s="16">
+      <c r="C6" s="15">
         <f>C5-Inputs!B35</f>
         <v>5</v>
       </c>
-      <c r="D6" s="16">
+      <c r="D6" s="15">
         <f>D5-Inputs!B35</f>
         <v>8</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>Michael's pot at retirement</t>
         </is>
       </c>
-      <c r="B7" s="18">
+      <c r="B7" s="17">
         <f>FV(Inputs!B23,B6,-Inputs!B41,-Inputs!B40,1)</f>
         <v>359817.718964</v>
       </c>
-      <c r="C7" s="18">
+      <c r="C7" s="17">
         <f>FV(Inputs!B23,C6,-Inputs!B41,-Inputs!B40,1)</f>
         <v>462361.886801</v>
       </c>
-      <c r="D7" s="18">
+      <c r="D7" s="17">
         <f>FV(Inputs!B23,D6,-Inputs!B41,-Inputs!B40,1)</f>
         <v>634140.15236</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>Michael's drawdown (~4%/yr)</t>
         </is>
       </c>
-      <c r="B8" s="18">
+      <c r="B8" s="17">
         <f>B7*Inputs!B26</f>
         <v>14392.708759</v>
       </c>
-      <c r="C8" s="18">
+      <c r="C8" s="17">
         <f>C7*Inputs!B26</f>
         <v>18494.475472</v>
       </c>
-      <c r="D8" s="18">
+      <c r="D8" s="17">
         <f>D7*Inputs!B26</f>
         <v>25365.606094</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>+ RAF pension</t>
         </is>
       </c>
-      <c r="B9" s="17">
+      <c r="B9" s="16">
         <f>Inputs!B53</f>
         <v>5340</v>
       </c>
-      <c r="C9" s="17">
+      <c r="C9" s="16">
         <f>Inputs!B53</f>
         <v>5340</v>
       </c>
-      <c r="D9" s="17">
+      <c r="D9" s="16">
         <f>Inputs!B53</f>
         <v>5340</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>+ State Pension</t>
         </is>
       </c>
-      <c r="B10" s="17">
+      <c r="B10" s="16">
         <f>Inputs!B39</f>
         <v>12532</v>
       </c>
-      <c r="C10" s="17">
+      <c r="C10" s="16">
         <f>Inputs!B39</f>
         <v>12532</v>
       </c>
-      <c r="D10" s="17">
+      <c r="D10" s="16">
         <f>Inputs!B39</f>
         <v>12532</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="22" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>Michael's total income /yr</t>
         </is>
       </c>
-      <c r="B11" s="29">
+      <c r="B11" s="28">
         <f>B8+B9+B10</f>
         <v>32264.708759</v>
       </c>
-      <c r="C11" s="29">
+      <c r="C11" s="28">
         <f>C8+C9+C10</f>
         <v>36366.475472</v>
       </c>
-      <c r="D11" s="29">
+      <c r="D11" s="28">
         <f>D8+D9+D10</f>
         <v>43237.606094</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Janey's total income /yr</t>
         </is>
       </c>
-      <c r="B12" s="17">
+      <c r="B12" s="16">
         <f>'Household'!B9</f>
-        <v>21281.677511</v>
-      </c>
-      <c r="C12" s="17">
+        <v>21808.677511</v>
+      </c>
+      <c r="C12" s="16">
         <f>'Household'!B9</f>
-        <v>21281.677511</v>
-      </c>
-      <c r="D12" s="17">
+        <v>21808.677511</v>
+      </c>
+      <c r="D12" s="16">
         <f>'Household'!B9</f>
-        <v>21281.677511</v>
+        <v>21808.677511</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="22" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>Household total /yr</t>
         </is>
       </c>
-      <c r="B13" s="23">
+      <c r="B13" s="22">
         <f>B11+B12</f>
-        <v>53546.38627</v>
-      </c>
-      <c r="C13" s="23">
+        <v>54073.38627</v>
+      </c>
+      <c r="C13" s="22">
         <f>C11+C12</f>
-        <v>57648.152983</v>
-      </c>
-      <c r="D13" s="23">
+        <v>58175.152983</v>
+      </c>
+      <c r="D13" s="22">
         <f>D11+D12</f>
-        <v>64519.283606</v>
+        <v>65046.283606</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>≈ per month</t>
         </is>
       </c>
-      <c r="B14" s="18">
+      <c r="B14" s="17">
         <f>B13/12</f>
-        <v>4462.198856</v>
-      </c>
-      <c r="C14" s="18">
+        <v>4506.115522</v>
+      </c>
+      <c r="C14" s="17">
         <f>C13/12</f>
-        <v>4804.012749</v>
-      </c>
-      <c r="D14" s="18">
+        <v>4847.929415</v>
+      </c>
+      <c r="D14" s="17">
         <f>D13/12</f>
-        <v>5376.606967</v>
+        <v>5420.523634</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>vs 'Comfortable' (£59,000)</t>
         </is>
       </c>
-      <c r="B15" s="25">
+      <c r="B15" s="24">
         <f>B13-59000</f>
-        <v>-5453.61373</v>
-      </c>
-      <c r="C15" s="25">
+        <v>-4926.61373</v>
+      </c>
+      <c r="C15" s="24">
         <f>C13-59000</f>
-        <v>-1351.847017</v>
-      </c>
-      <c r="D15" s="25">
+        <v>-824.847017</v>
+      </c>
+      <c r="D15" s="24">
         <f>D13-59000</f>
-        <v>5519.283606</v>
+        <v>6046.283606</v>
       </c>
     </row>
     <row r="17">
@@ -3514,7 +3513,7 @@
       </c>
       <c r="B8" s="8">
         <f>'Household'!D9</f>
-        <v>64519.283606</v>
+        <v>65046.283606</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -3539,9 +3538,9 @@
           <t>Household income — Comfortable-plus /yr</t>
         </is>
       </c>
-      <c r="B10" s="19">
+      <c r="B10" s="18">
         <f>B8+B9</f>
-        <v>67192.832758</v>
+        <v>67719.832758</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -3557,7 +3556,7 @@
       </c>
       <c r="B11" s="8">
         <f>B10/12</f>
-        <v>5599.40273</v>
+        <v>5643.319396</v>
       </c>
     </row>
     <row r="12">
@@ -3566,9 +3565,9 @@
           <t>vs 'Comfortable' (£59,000)</t>
         </is>
       </c>
-      <c r="B12" s="30">
+      <c r="B12" s="29">
         <f>B10-59000</f>
-        <v>8192.832758</v>
+        <v>8719.832758</v>
       </c>
     </row>
     <row r="14">

</xml_diff>